<commit_message>
feat: support challenge positions and expand authoring guides
Carry optional positions through XLSX/CSV validation, manifest export, dry-run previews, and atomic imports while preserving legacy inputs and blank-value semantics.

Regenerate the workbook, add ordering regression coverage, and document all authoring fields, dynamic scoring, and first-solver bonus tiers.
</commit_message>
<xml_diff>
--- a/tools/push-challenges-template.xlsx
+++ b/tools/push-challenges-template.xlsx
@@ -160,9 +160,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChallengesTable" displayName="ChallengesTable" ref="A1:P501" headerRowCount="1">
-  <autoFilter ref="A1:P501"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChallengesTable" displayName="ChallengesTable" ref="A1:Q501" headerRowCount="1">
+  <autoFilter ref="A1:Q501"/>
+  <tableColumns count="17">
     <tableColumn id="1" name="Name"/>
     <tableColumn id="2" name="Description"/>
     <tableColumn id="3" name="Value"/>
@@ -179,6 +179,7 @@
     <tableColumn id="14" name="Minimum Value"/>
     <tableColumn id="15" name="Decay"/>
     <tableColumn id="16" name="Bonus Mode"/>
+    <tableColumn id="17" name="Position"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -525,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -637,6 +638,18 @@
       <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Existing Standard/Dynamic type mismatches skip only that challenge. Review MANUAL ACTION REQUIRED at the end of every import. Change types manually in CTFd and rerun. Files remain manual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Optional display order: positive whole numbers sort lowest first. 0 uses CTFd automatic point ordering. Blank preserves an existing position or leaves a new challenge at 0. Next is navigation, not order.</t>
         </is>
       </c>
     </row>
@@ -651,7 +664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P501"/>
+  <dimension ref="A1:Q501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -670,6 +683,7 @@
     <col width="18" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -751,6 +765,11 @@
       <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Bonus Mode</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>Position</t>
         </is>
       </c>
     </row>
@@ -785,6 +804,7 @@
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n"/>
@@ -817,6 +837,7 @@
       <c r="N3" s="2" t="n"/>
       <c r="O3" s="2" t="n"/>
       <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n"/>
@@ -849,6 +870,7 @@
       <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="n"/>
+      <c r="Q4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n"/>
@@ -881,6 +903,7 @@
       <c r="N5" s="2" t="n"/>
       <c r="O5" s="2" t="n"/>
       <c r="P5" s="2" t="n"/>
+      <c r="Q5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n"/>
@@ -913,6 +936,7 @@
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="n"/>
       <c r="P6" s="2" t="n"/>
+      <c r="Q6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n"/>
@@ -945,6 +969,7 @@
       <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="n"/>
       <c r="P7" s="2" t="n"/>
+      <c r="Q7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
@@ -977,6 +1002,7 @@
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="n"/>
       <c r="P8" s="2" t="n"/>
+      <c r="Q8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n"/>
@@ -1009,6 +1035,7 @@
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="n"/>
+      <c r="Q9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
@@ -1041,6 +1068,7 @@
       <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="n"/>
       <c r="P10" s="2" t="n"/>
+      <c r="Q10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>
@@ -1073,6 +1101,7 @@
       <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="n"/>
       <c r="P11" s="2" t="n"/>
+      <c r="Q11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
@@ -1105,6 +1134,7 @@
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="n"/>
+      <c r="Q12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -1137,6 +1167,7 @@
       <c r="N13" s="2" t="n"/>
       <c r="O13" s="2" t="n"/>
       <c r="P13" s="2" t="n"/>
+      <c r="Q13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -1169,6 +1200,7 @@
       <c r="N14" s="2" t="n"/>
       <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="n"/>
+      <c r="Q14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
@@ -1201,6 +1233,7 @@
       <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="n"/>
       <c r="P15" s="2" t="n"/>
+      <c r="Q15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
@@ -1233,6 +1266,7 @@
       <c r="N16" s="2" t="n"/>
       <c r="O16" s="2" t="n"/>
       <c r="P16" s="2" t="n"/>
+      <c r="Q16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
@@ -1265,6 +1299,7 @@
       <c r="N17" s="2" t="n"/>
       <c r="O17" s="2" t="n"/>
       <c r="P17" s="2" t="n"/>
+      <c r="Q17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
@@ -1297,6 +1332,7 @@
       <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="n"/>
       <c r="P18" s="2" t="n"/>
+      <c r="Q18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
@@ -1329,6 +1365,7 @@
       <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="n"/>
       <c r="P19" s="2" t="n"/>
+      <c r="Q19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
@@ -1361,6 +1398,7 @@
       <c r="N20" s="2" t="n"/>
       <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="n"/>
+      <c r="Q20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
@@ -1393,6 +1431,7 @@
       <c r="N21" s="2" t="n"/>
       <c r="O21" s="2" t="n"/>
       <c r="P21" s="2" t="n"/>
+      <c r="Q21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
@@ -1425,6 +1464,7 @@
       <c r="N22" s="2" t="n"/>
       <c r="O22" s="2" t="n"/>
       <c r="P22" s="2" t="n"/>
+      <c r="Q22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
@@ -1457,6 +1497,7 @@
       <c r="N23" s="2" t="n"/>
       <c r="O23" s="2" t="n"/>
       <c r="P23" s="2" t="n"/>
+      <c r="Q23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
@@ -1489,6 +1530,7 @@
       <c r="N24" s="2" t="n"/>
       <c r="O24" s="2" t="n"/>
       <c r="P24" s="2" t="n"/>
+      <c r="Q24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
@@ -1521,6 +1563,7 @@
       <c r="N25" s="2" t="n"/>
       <c r="O25" s="2" t="n"/>
       <c r="P25" s="2" t="n"/>
+      <c r="Q25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
@@ -1553,6 +1596,7 @@
       <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="n"/>
+      <c r="Q26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
@@ -1585,6 +1629,7 @@
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="n"/>
       <c r="P27" s="2" t="n"/>
+      <c r="Q27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
@@ -1617,6 +1662,7 @@
       <c r="N28" s="2" t="n"/>
       <c r="O28" s="2" t="n"/>
       <c r="P28" s="2" t="n"/>
+      <c r="Q28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
@@ -1649,6 +1695,7 @@
       <c r="N29" s="2" t="n"/>
       <c r="O29" s="2" t="n"/>
       <c r="P29" s="2" t="n"/>
+      <c r="Q29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
@@ -1681,6 +1728,7 @@
       <c r="N30" s="2" t="n"/>
       <c r="O30" s="2" t="n"/>
       <c r="P30" s="2" t="n"/>
+      <c r="Q30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
@@ -1713,6 +1761,7 @@
       <c r="N31" s="2" t="n"/>
       <c r="O31" s="2" t="n"/>
       <c r="P31" s="2" t="n"/>
+      <c r="Q31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n"/>
@@ -1745,6 +1794,7 @@
       <c r="N32" s="2" t="n"/>
       <c r="O32" s="2" t="n"/>
       <c r="P32" s="2" t="n"/>
+      <c r="Q32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n"/>
@@ -1777,6 +1827,7 @@
       <c r="N33" s="2" t="n"/>
       <c r="O33" s="2" t="n"/>
       <c r="P33" s="2" t="n"/>
+      <c r="Q33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n"/>
@@ -1809,6 +1860,7 @@
       <c r="N34" s="2" t="n"/>
       <c r="O34" s="2" t="n"/>
       <c r="P34" s="2" t="n"/>
+      <c r="Q34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>
@@ -1841,6 +1893,7 @@
       <c r="N35" s="2" t="n"/>
       <c r="O35" s="2" t="n"/>
       <c r="P35" s="2" t="n"/>
+      <c r="Q35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
@@ -1873,6 +1926,7 @@
       <c r="N36" s="2" t="n"/>
       <c r="O36" s="2" t="n"/>
       <c r="P36" s="2" t="n"/>
+      <c r="Q36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
@@ -1905,6 +1959,7 @@
       <c r="N37" s="2" t="n"/>
       <c r="O37" s="2" t="n"/>
       <c r="P37" s="2" t="n"/>
+      <c r="Q37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
@@ -1937,6 +1992,7 @@
       <c r="N38" s="2" t="n"/>
       <c r="O38" s="2" t="n"/>
       <c r="P38" s="2" t="n"/>
+      <c r="Q38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
@@ -1969,6 +2025,7 @@
       <c r="N39" s="2" t="n"/>
       <c r="O39" s="2" t="n"/>
       <c r="P39" s="2" t="n"/>
+      <c r="Q39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
@@ -2001,6 +2058,7 @@
       <c r="N40" s="2" t="n"/>
       <c r="O40" s="2" t="n"/>
       <c r="P40" s="2" t="n"/>
+      <c r="Q40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
@@ -2033,6 +2091,7 @@
       <c r="N41" s="2" t="n"/>
       <c r="O41" s="2" t="n"/>
       <c r="P41" s="2" t="n"/>
+      <c r="Q41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
@@ -2065,6 +2124,7 @@
       <c r="N42" s="2" t="n"/>
       <c r="O42" s="2" t="n"/>
       <c r="P42" s="2" t="n"/>
+      <c r="Q42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
@@ -2097,6 +2157,7 @@
       <c r="N43" s="2" t="n"/>
       <c r="O43" s="2" t="n"/>
       <c r="P43" s="2" t="n"/>
+      <c r="Q43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
@@ -2129,6 +2190,7 @@
       <c r="N44" s="2" t="n"/>
       <c r="O44" s="2" t="n"/>
       <c r="P44" s="2" t="n"/>
+      <c r="Q44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
@@ -2161,6 +2223,7 @@
       <c r="N45" s="2" t="n"/>
       <c r="O45" s="2" t="n"/>
       <c r="P45" s="2" t="n"/>
+      <c r="Q45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
@@ -2193,6 +2256,7 @@
       <c r="N46" s="2" t="n"/>
       <c r="O46" s="2" t="n"/>
       <c r="P46" s="2" t="n"/>
+      <c r="Q46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
@@ -2225,6 +2289,7 @@
       <c r="N47" s="2" t="n"/>
       <c r="O47" s="2" t="n"/>
       <c r="P47" s="2" t="n"/>
+      <c r="Q47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -2257,6 +2322,7 @@
       <c r="N48" s="2" t="n"/>
       <c r="O48" s="2" t="n"/>
       <c r="P48" s="2" t="n"/>
+      <c r="Q48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
@@ -2289,6 +2355,7 @@
       <c r="N49" s="2" t="n"/>
       <c r="O49" s="2" t="n"/>
       <c r="P49" s="2" t="n"/>
+      <c r="Q49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
@@ -2321,6 +2388,7 @@
       <c r="N50" s="2" t="n"/>
       <c r="O50" s="2" t="n"/>
       <c r="P50" s="2" t="n"/>
+      <c r="Q50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
@@ -2353,6 +2421,7 @@
       <c r="N51" s="2" t="n"/>
       <c r="O51" s="2" t="n"/>
       <c r="P51" s="2" t="n"/>
+      <c r="Q51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
@@ -2385,6 +2454,7 @@
       <c r="N52" s="2" t="n"/>
       <c r="O52" s="2" t="n"/>
       <c r="P52" s="2" t="n"/>
+      <c r="Q52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n"/>
@@ -2417,6 +2487,7 @@
       <c r="N53" s="2" t="n"/>
       <c r="O53" s="2" t="n"/>
       <c r="P53" s="2" t="n"/>
+      <c r="Q53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
@@ -2449,6 +2520,7 @@
       <c r="N54" s="2" t="n"/>
       <c r="O54" s="2" t="n"/>
       <c r="P54" s="2" t="n"/>
+      <c r="Q54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
@@ -2481,6 +2553,7 @@
       <c r="N55" s="2" t="n"/>
       <c r="O55" s="2" t="n"/>
       <c r="P55" s="2" t="n"/>
+      <c r="Q55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
@@ -2513,6 +2586,7 @@
       <c r="N56" s="2" t="n"/>
       <c r="O56" s="2" t="n"/>
       <c r="P56" s="2" t="n"/>
+      <c r="Q56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
@@ -2545,6 +2619,7 @@
       <c r="N57" s="2" t="n"/>
       <c r="O57" s="2" t="n"/>
       <c r="P57" s="2" t="n"/>
+      <c r="Q57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
@@ -2577,6 +2652,7 @@
       <c r="N58" s="2" t="n"/>
       <c r="O58" s="2" t="n"/>
       <c r="P58" s="2" t="n"/>
+      <c r="Q58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
@@ -2609,6 +2685,7 @@
       <c r="N59" s="2" t="n"/>
       <c r="O59" s="2" t="n"/>
       <c r="P59" s="2" t="n"/>
+      <c r="Q59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
@@ -2641,6 +2718,7 @@
       <c r="N60" s="2" t="n"/>
       <c r="O60" s="2" t="n"/>
       <c r="P60" s="2" t="n"/>
+      <c r="Q60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
@@ -2673,6 +2751,7 @@
       <c r="N61" s="2" t="n"/>
       <c r="O61" s="2" t="n"/>
       <c r="P61" s="2" t="n"/>
+      <c r="Q61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
@@ -2705,6 +2784,7 @@
       <c r="N62" s="2" t="n"/>
       <c r="O62" s="2" t="n"/>
       <c r="P62" s="2" t="n"/>
+      <c r="Q62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>
@@ -2737,6 +2817,7 @@
       <c r="N63" s="2" t="n"/>
       <c r="O63" s="2" t="n"/>
       <c r="P63" s="2" t="n"/>
+      <c r="Q63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>
@@ -2769,6 +2850,7 @@
       <c r="N64" s="2" t="n"/>
       <c r="O64" s="2" t="n"/>
       <c r="P64" s="2" t="n"/>
+      <c r="Q64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
@@ -2801,6 +2883,7 @@
       <c r="N65" s="2" t="n"/>
       <c r="O65" s="2" t="n"/>
       <c r="P65" s="2" t="n"/>
+      <c r="Q65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
@@ -2833,6 +2916,7 @@
       <c r="N66" s="2" t="n"/>
       <c r="O66" s="2" t="n"/>
       <c r="P66" s="2" t="n"/>
+      <c r="Q66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
@@ -2865,6 +2949,7 @@
       <c r="N67" s="2" t="n"/>
       <c r="O67" s="2" t="n"/>
       <c r="P67" s="2" t="n"/>
+      <c r="Q67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n"/>
@@ -2897,6 +2982,7 @@
       <c r="N68" s="2" t="n"/>
       <c r="O68" s="2" t="n"/>
       <c r="P68" s="2" t="n"/>
+      <c r="Q68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
@@ -2929,6 +3015,7 @@
       <c r="N69" s="2" t="n"/>
       <c r="O69" s="2" t="n"/>
       <c r="P69" s="2" t="n"/>
+      <c r="Q69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
@@ -2961,6 +3048,7 @@
       <c r="N70" s="2" t="n"/>
       <c r="O70" s="2" t="n"/>
       <c r="P70" s="2" t="n"/>
+      <c r="Q70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
@@ -2993,6 +3081,7 @@
       <c r="N71" s="2" t="n"/>
       <c r="O71" s="2" t="n"/>
       <c r="P71" s="2" t="n"/>
+      <c r="Q71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
@@ -3025,6 +3114,7 @@
       <c r="N72" s="2" t="n"/>
       <c r="O72" s="2" t="n"/>
       <c r="P72" s="2" t="n"/>
+      <c r="Q72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
@@ -3057,6 +3147,7 @@
       <c r="N73" s="2" t="n"/>
       <c r="O73" s="2" t="n"/>
       <c r="P73" s="2" t="n"/>
+      <c r="Q73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
@@ -3089,6 +3180,7 @@
       <c r="N74" s="2" t="n"/>
       <c r="O74" s="2" t="n"/>
       <c r="P74" s="2" t="n"/>
+      <c r="Q74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
@@ -3121,6 +3213,7 @@
       <c r="N75" s="2" t="n"/>
       <c r="O75" s="2" t="n"/>
       <c r="P75" s="2" t="n"/>
+      <c r="Q75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n"/>
@@ -3153,6 +3246,7 @@
       <c r="N76" s="2" t="n"/>
       <c r="O76" s="2" t="n"/>
       <c r="P76" s="2" t="n"/>
+      <c r="Q76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
@@ -3185,6 +3279,7 @@
       <c r="N77" s="2" t="n"/>
       <c r="O77" s="2" t="n"/>
       <c r="P77" s="2" t="n"/>
+      <c r="Q77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
@@ -3217,6 +3312,7 @@
       <c r="N78" s="2" t="n"/>
       <c r="O78" s="2" t="n"/>
       <c r="P78" s="2" t="n"/>
+      <c r="Q78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
@@ -3249,6 +3345,7 @@
       <c r="N79" s="2" t="n"/>
       <c r="O79" s="2" t="n"/>
       <c r="P79" s="2" t="n"/>
+      <c r="Q79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
@@ -3281,6 +3378,7 @@
       <c r="N80" s="2" t="n"/>
       <c r="O80" s="2" t="n"/>
       <c r="P80" s="2" t="n"/>
+      <c r="Q80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
@@ -3313,6 +3411,7 @@
       <c r="N81" s="2" t="n"/>
       <c r="O81" s="2" t="n"/>
       <c r="P81" s="2" t="n"/>
+      <c r="Q81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
@@ -3345,6 +3444,7 @@
       <c r="N82" s="2" t="n"/>
       <c r="O82" s="2" t="n"/>
       <c r="P82" s="2" t="n"/>
+      <c r="Q82" s="2" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
@@ -3377,6 +3477,7 @@
       <c r="N83" s="2" t="n"/>
       <c r="O83" s="2" t="n"/>
       <c r="P83" s="2" t="n"/>
+      <c r="Q83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
@@ -3409,6 +3510,7 @@
       <c r="N84" s="2" t="n"/>
       <c r="O84" s="2" t="n"/>
       <c r="P84" s="2" t="n"/>
+      <c r="Q84" s="2" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n"/>
@@ -3441,6 +3543,7 @@
       <c r="N85" s="2" t="n"/>
       <c r="O85" s="2" t="n"/>
       <c r="P85" s="2" t="n"/>
+      <c r="Q85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n"/>
@@ -3473,6 +3576,7 @@
       <c r="N86" s="2" t="n"/>
       <c r="O86" s="2" t="n"/>
       <c r="P86" s="2" t="n"/>
+      <c r="Q86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n"/>
@@ -3505,6 +3609,7 @@
       <c r="N87" s="2" t="n"/>
       <c r="O87" s="2" t="n"/>
       <c r="P87" s="2" t="n"/>
+      <c r="Q87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
@@ -3537,6 +3642,7 @@
       <c r="N88" s="2" t="n"/>
       <c r="O88" s="2" t="n"/>
       <c r="P88" s="2" t="n"/>
+      <c r="Q88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n"/>
@@ -3569,6 +3675,7 @@
       <c r="N89" s="2" t="n"/>
       <c r="O89" s="2" t="n"/>
       <c r="P89" s="2" t="n"/>
+      <c r="Q89" s="2" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n"/>
@@ -3601,6 +3708,7 @@
       <c r="N90" s="2" t="n"/>
       <c r="O90" s="2" t="n"/>
       <c r="P90" s="2" t="n"/>
+      <c r="Q90" s="2" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n"/>
@@ -3633,6 +3741,7 @@
       <c r="N91" s="2" t="n"/>
       <c r="O91" s="2" t="n"/>
       <c r="P91" s="2" t="n"/>
+      <c r="Q91" s="2" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n"/>
@@ -3665,6 +3774,7 @@
       <c r="N92" s="2" t="n"/>
       <c r="O92" s="2" t="n"/>
       <c r="P92" s="2" t="n"/>
+      <c r="Q92" s="2" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n"/>
@@ -3697,6 +3807,7 @@
       <c r="N93" s="2" t="n"/>
       <c r="O93" s="2" t="n"/>
       <c r="P93" s="2" t="n"/>
+      <c r="Q93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n"/>
@@ -3729,6 +3840,7 @@
       <c r="N94" s="2" t="n"/>
       <c r="O94" s="2" t="n"/>
       <c r="P94" s="2" t="n"/>
+      <c r="Q94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n"/>
@@ -3761,6 +3873,7 @@
       <c r="N95" s="2" t="n"/>
       <c r="O95" s="2" t="n"/>
       <c r="P95" s="2" t="n"/>
+      <c r="Q95" s="2" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n"/>
@@ -3793,6 +3906,7 @@
       <c r="N96" s="2" t="n"/>
       <c r="O96" s="2" t="n"/>
       <c r="P96" s="2" t="n"/>
+      <c r="Q96" s="2" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n"/>
@@ -3825,6 +3939,7 @@
       <c r="N97" s="2" t="n"/>
       <c r="O97" s="2" t="n"/>
       <c r="P97" s="2" t="n"/>
+      <c r="Q97" s="2" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n"/>
@@ -3857,6 +3972,7 @@
       <c r="N98" s="2" t="n"/>
       <c r="O98" s="2" t="n"/>
       <c r="P98" s="2" t="n"/>
+      <c r="Q98" s="2" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n"/>
@@ -3889,6 +4005,7 @@
       <c r="N99" s="2" t="n"/>
       <c r="O99" s="2" t="n"/>
       <c r="P99" s="2" t="n"/>
+      <c r="Q99" s="2" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n"/>
@@ -3921,6 +4038,7 @@
       <c r="N100" s="2" t="n"/>
       <c r="O100" s="2" t="n"/>
       <c r="P100" s="2" t="n"/>
+      <c r="Q100" s="2" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n"/>
@@ -3953,6 +4071,7 @@
       <c r="N101" s="2" t="n"/>
       <c r="O101" s="2" t="n"/>
       <c r="P101" s="2" t="n"/>
+      <c r="Q101" s="2" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n"/>
@@ -3985,6 +4104,7 @@
       <c r="N102" s="2" t="n"/>
       <c r="O102" s="2" t="n"/>
       <c r="P102" s="2" t="n"/>
+      <c r="Q102" s="2" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n"/>
@@ -4017,6 +4137,7 @@
       <c r="N103" s="2" t="n"/>
       <c r="O103" s="2" t="n"/>
       <c r="P103" s="2" t="n"/>
+      <c r="Q103" s="2" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n"/>
@@ -4049,6 +4170,7 @@
       <c r="N104" s="2" t="n"/>
       <c r="O104" s="2" t="n"/>
       <c r="P104" s="2" t="n"/>
+      <c r="Q104" s="2" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n"/>
@@ -4081,6 +4203,7 @@
       <c r="N105" s="2" t="n"/>
       <c r="O105" s="2" t="n"/>
       <c r="P105" s="2" t="n"/>
+      <c r="Q105" s="2" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n"/>
@@ -4113,6 +4236,7 @@
       <c r="N106" s="2" t="n"/>
       <c r="O106" s="2" t="n"/>
       <c r="P106" s="2" t="n"/>
+      <c r="Q106" s="2" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n"/>
@@ -4145,6 +4269,7 @@
       <c r="N107" s="2" t="n"/>
       <c r="O107" s="2" t="n"/>
       <c r="P107" s="2" t="n"/>
+      <c r="Q107" s="2" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n"/>
@@ -4177,6 +4302,7 @@
       <c r="N108" s="2" t="n"/>
       <c r="O108" s="2" t="n"/>
       <c r="P108" s="2" t="n"/>
+      <c r="Q108" s="2" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n"/>
@@ -4209,6 +4335,7 @@
       <c r="N109" s="2" t="n"/>
       <c r="O109" s="2" t="n"/>
       <c r="P109" s="2" t="n"/>
+      <c r="Q109" s="2" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n"/>
@@ -4241,6 +4368,7 @@
       <c r="N110" s="2" t="n"/>
       <c r="O110" s="2" t="n"/>
       <c r="P110" s="2" t="n"/>
+      <c r="Q110" s="2" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n"/>
@@ -4273,6 +4401,7 @@
       <c r="N111" s="2" t="n"/>
       <c r="O111" s="2" t="n"/>
       <c r="P111" s="2" t="n"/>
+      <c r="Q111" s="2" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n"/>
@@ -4305,6 +4434,7 @@
       <c r="N112" s="2" t="n"/>
       <c r="O112" s="2" t="n"/>
       <c r="P112" s="2" t="n"/>
+      <c r="Q112" s="2" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n"/>
@@ -4337,6 +4467,7 @@
       <c r="N113" s="2" t="n"/>
       <c r="O113" s="2" t="n"/>
       <c r="P113" s="2" t="n"/>
+      <c r="Q113" s="2" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n"/>
@@ -4369,6 +4500,7 @@
       <c r="N114" s="2" t="n"/>
       <c r="O114" s="2" t="n"/>
       <c r="P114" s="2" t="n"/>
+      <c r="Q114" s="2" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n"/>
@@ -4401,6 +4533,7 @@
       <c r="N115" s="2" t="n"/>
       <c r="O115" s="2" t="n"/>
       <c r="P115" s="2" t="n"/>
+      <c r="Q115" s="2" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n"/>
@@ -4433,6 +4566,7 @@
       <c r="N116" s="2" t="n"/>
       <c r="O116" s="2" t="n"/>
       <c r="P116" s="2" t="n"/>
+      <c r="Q116" s="2" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n"/>
@@ -4465,6 +4599,7 @@
       <c r="N117" s="2" t="n"/>
       <c r="O117" s="2" t="n"/>
       <c r="P117" s="2" t="n"/>
+      <c r="Q117" s="2" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n"/>
@@ -4497,6 +4632,7 @@
       <c r="N118" s="2" t="n"/>
       <c r="O118" s="2" t="n"/>
       <c r="P118" s="2" t="n"/>
+      <c r="Q118" s="2" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n"/>
@@ -4529,6 +4665,7 @@
       <c r="N119" s="2" t="n"/>
       <c r="O119" s="2" t="n"/>
       <c r="P119" s="2" t="n"/>
+      <c r="Q119" s="2" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n"/>
@@ -4561,6 +4698,7 @@
       <c r="N120" s="2" t="n"/>
       <c r="O120" s="2" t="n"/>
       <c r="P120" s="2" t="n"/>
+      <c r="Q120" s="2" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n"/>
@@ -4593,6 +4731,7 @@
       <c r="N121" s="2" t="n"/>
       <c r="O121" s="2" t="n"/>
       <c r="P121" s="2" t="n"/>
+      <c r="Q121" s="2" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n"/>
@@ -4625,6 +4764,7 @@
       <c r="N122" s="2" t="n"/>
       <c r="O122" s="2" t="n"/>
       <c r="P122" s="2" t="n"/>
+      <c r="Q122" s="2" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n"/>
@@ -4657,6 +4797,7 @@
       <c r="N123" s="2" t="n"/>
       <c r="O123" s="2" t="n"/>
       <c r="P123" s="2" t="n"/>
+      <c r="Q123" s="2" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n"/>
@@ -4689,6 +4830,7 @@
       <c r="N124" s="2" t="n"/>
       <c r="O124" s="2" t="n"/>
       <c r="P124" s="2" t="n"/>
+      <c r="Q124" s="2" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n"/>
@@ -4721,6 +4863,7 @@
       <c r="N125" s="2" t="n"/>
       <c r="O125" s="2" t="n"/>
       <c r="P125" s="2" t="n"/>
+      <c r="Q125" s="2" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n"/>
@@ -4753,6 +4896,7 @@
       <c r="N126" s="2" t="n"/>
       <c r="O126" s="2" t="n"/>
       <c r="P126" s="2" t="n"/>
+      <c r="Q126" s="2" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n"/>
@@ -4785,6 +4929,7 @@
       <c r="N127" s="2" t="n"/>
       <c r="O127" s="2" t="n"/>
       <c r="P127" s="2" t="n"/>
+      <c r="Q127" s="2" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n"/>
@@ -4817,6 +4962,7 @@
       <c r="N128" s="2" t="n"/>
       <c r="O128" s="2" t="n"/>
       <c r="P128" s="2" t="n"/>
+      <c r="Q128" s="2" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n"/>
@@ -4849,6 +4995,7 @@
       <c r="N129" s="2" t="n"/>
       <c r="O129" s="2" t="n"/>
       <c r="P129" s="2" t="n"/>
+      <c r="Q129" s="2" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n"/>
@@ -4881,6 +5028,7 @@
       <c r="N130" s="2" t="n"/>
       <c r="O130" s="2" t="n"/>
       <c r="P130" s="2" t="n"/>
+      <c r="Q130" s="2" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n"/>
@@ -4913,6 +5061,7 @@
       <c r="N131" s="2" t="n"/>
       <c r="O131" s="2" t="n"/>
       <c r="P131" s="2" t="n"/>
+      <c r="Q131" s="2" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n"/>
@@ -4945,6 +5094,7 @@
       <c r="N132" s="2" t="n"/>
       <c r="O132" s="2" t="n"/>
       <c r="P132" s="2" t="n"/>
+      <c r="Q132" s="2" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n"/>
@@ -4977,6 +5127,7 @@
       <c r="N133" s="2" t="n"/>
       <c r="O133" s="2" t="n"/>
       <c r="P133" s="2" t="n"/>
+      <c r="Q133" s="2" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n"/>
@@ -5009,6 +5160,7 @@
       <c r="N134" s="2" t="n"/>
       <c r="O134" s="2" t="n"/>
       <c r="P134" s="2" t="n"/>
+      <c r="Q134" s="2" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n"/>
@@ -5041,6 +5193,7 @@
       <c r="N135" s="2" t="n"/>
       <c r="O135" s="2" t="n"/>
       <c r="P135" s="2" t="n"/>
+      <c r="Q135" s="2" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n"/>
@@ -5073,6 +5226,7 @@
       <c r="N136" s="2" t="n"/>
       <c r="O136" s="2" t="n"/>
       <c r="P136" s="2" t="n"/>
+      <c r="Q136" s="2" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n"/>
@@ -5105,6 +5259,7 @@
       <c r="N137" s="2" t="n"/>
       <c r="O137" s="2" t="n"/>
       <c r="P137" s="2" t="n"/>
+      <c r="Q137" s="2" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n"/>
@@ -5137,6 +5292,7 @@
       <c r="N138" s="2" t="n"/>
       <c r="O138" s="2" t="n"/>
       <c r="P138" s="2" t="n"/>
+      <c r="Q138" s="2" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n"/>
@@ -5169,6 +5325,7 @@
       <c r="N139" s="2" t="n"/>
       <c r="O139" s="2" t="n"/>
       <c r="P139" s="2" t="n"/>
+      <c r="Q139" s="2" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n"/>
@@ -5201,6 +5358,7 @@
       <c r="N140" s="2" t="n"/>
       <c r="O140" s="2" t="n"/>
       <c r="P140" s="2" t="n"/>
+      <c r="Q140" s="2" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n"/>
@@ -5233,6 +5391,7 @@
       <c r="N141" s="2" t="n"/>
       <c r="O141" s="2" t="n"/>
       <c r="P141" s="2" t="n"/>
+      <c r="Q141" s="2" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n"/>
@@ -5265,6 +5424,7 @@
       <c r="N142" s="2" t="n"/>
       <c r="O142" s="2" t="n"/>
       <c r="P142" s="2" t="n"/>
+      <c r="Q142" s="2" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n"/>
@@ -5297,6 +5457,7 @@
       <c r="N143" s="2" t="n"/>
       <c r="O143" s="2" t="n"/>
       <c r="P143" s="2" t="n"/>
+      <c r="Q143" s="2" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n"/>
@@ -5329,6 +5490,7 @@
       <c r="N144" s="2" t="n"/>
       <c r="O144" s="2" t="n"/>
       <c r="P144" s="2" t="n"/>
+      <c r="Q144" s="2" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n"/>
@@ -5361,6 +5523,7 @@
       <c r="N145" s="2" t="n"/>
       <c r="O145" s="2" t="n"/>
       <c r="P145" s="2" t="n"/>
+      <c r="Q145" s="2" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n"/>
@@ -5393,6 +5556,7 @@
       <c r="N146" s="2" t="n"/>
       <c r="O146" s="2" t="n"/>
       <c r="P146" s="2" t="n"/>
+      <c r="Q146" s="2" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n"/>
@@ -5425,6 +5589,7 @@
       <c r="N147" s="2" t="n"/>
       <c r="O147" s="2" t="n"/>
       <c r="P147" s="2" t="n"/>
+      <c r="Q147" s="2" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n"/>
@@ -5457,6 +5622,7 @@
       <c r="N148" s="2" t="n"/>
       <c r="O148" s="2" t="n"/>
       <c r="P148" s="2" t="n"/>
+      <c r="Q148" s="2" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n"/>
@@ -5489,6 +5655,7 @@
       <c r="N149" s="2" t="n"/>
       <c r="O149" s="2" t="n"/>
       <c r="P149" s="2" t="n"/>
+      <c r="Q149" s="2" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n"/>
@@ -5521,6 +5688,7 @@
       <c r="N150" s="2" t="n"/>
       <c r="O150" s="2" t="n"/>
       <c r="P150" s="2" t="n"/>
+      <c r="Q150" s="2" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n"/>
@@ -5553,6 +5721,7 @@
       <c r="N151" s="2" t="n"/>
       <c r="O151" s="2" t="n"/>
       <c r="P151" s="2" t="n"/>
+      <c r="Q151" s="2" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n"/>
@@ -5585,6 +5754,7 @@
       <c r="N152" s="2" t="n"/>
       <c r="O152" s="2" t="n"/>
       <c r="P152" s="2" t="n"/>
+      <c r="Q152" s="2" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="n"/>
@@ -5617,6 +5787,7 @@
       <c r="N153" s="2" t="n"/>
       <c r="O153" s="2" t="n"/>
       <c r="P153" s="2" t="n"/>
+      <c r="Q153" s="2" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n"/>
@@ -5649,6 +5820,7 @@
       <c r="N154" s="2" t="n"/>
       <c r="O154" s="2" t="n"/>
       <c r="P154" s="2" t="n"/>
+      <c r="Q154" s="2" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n"/>
@@ -5681,6 +5853,7 @@
       <c r="N155" s="2" t="n"/>
       <c r="O155" s="2" t="n"/>
       <c r="P155" s="2" t="n"/>
+      <c r="Q155" s="2" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n"/>
@@ -5713,6 +5886,7 @@
       <c r="N156" s="2" t="n"/>
       <c r="O156" s="2" t="n"/>
       <c r="P156" s="2" t="n"/>
+      <c r="Q156" s="2" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n"/>
@@ -5745,6 +5919,7 @@
       <c r="N157" s="2" t="n"/>
       <c r="O157" s="2" t="n"/>
       <c r="P157" s="2" t="n"/>
+      <c r="Q157" s="2" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n"/>
@@ -5777,6 +5952,7 @@
       <c r="N158" s="2" t="n"/>
       <c r="O158" s="2" t="n"/>
       <c r="P158" s="2" t="n"/>
+      <c r="Q158" s="2" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n"/>
@@ -5809,6 +5985,7 @@
       <c r="N159" s="2" t="n"/>
       <c r="O159" s="2" t="n"/>
       <c r="P159" s="2" t="n"/>
+      <c r="Q159" s="2" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n"/>
@@ -5841,6 +6018,7 @@
       <c r="N160" s="2" t="n"/>
       <c r="O160" s="2" t="n"/>
       <c r="P160" s="2" t="n"/>
+      <c r="Q160" s="2" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="n"/>
@@ -5873,6 +6051,7 @@
       <c r="N161" s="2" t="n"/>
       <c r="O161" s="2" t="n"/>
       <c r="P161" s="2" t="n"/>
+      <c r="Q161" s="2" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n"/>
@@ -5905,6 +6084,7 @@
       <c r="N162" s="2" t="n"/>
       <c r="O162" s="2" t="n"/>
       <c r="P162" s="2" t="n"/>
+      <c r="Q162" s="2" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n"/>
@@ -5937,6 +6117,7 @@
       <c r="N163" s="2" t="n"/>
       <c r="O163" s="2" t="n"/>
       <c r="P163" s="2" t="n"/>
+      <c r="Q163" s="2" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n"/>
@@ -5969,6 +6150,7 @@
       <c r="N164" s="2" t="n"/>
       <c r="O164" s="2" t="n"/>
       <c r="P164" s="2" t="n"/>
+      <c r="Q164" s="2" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n"/>
@@ -6001,6 +6183,7 @@
       <c r="N165" s="2" t="n"/>
       <c r="O165" s="2" t="n"/>
       <c r="P165" s="2" t="n"/>
+      <c r="Q165" s="2" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n"/>
@@ -6033,6 +6216,7 @@
       <c r="N166" s="2" t="n"/>
       <c r="O166" s="2" t="n"/>
       <c r="P166" s="2" t="n"/>
+      <c r="Q166" s="2" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n"/>
@@ -6065,6 +6249,7 @@
       <c r="N167" s="2" t="n"/>
       <c r="O167" s="2" t="n"/>
       <c r="P167" s="2" t="n"/>
+      <c r="Q167" s="2" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n"/>
@@ -6097,6 +6282,7 @@
       <c r="N168" s="2" t="n"/>
       <c r="O168" s="2" t="n"/>
       <c r="P168" s="2" t="n"/>
+      <c r="Q168" s="2" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n"/>
@@ -6129,6 +6315,7 @@
       <c r="N169" s="2" t="n"/>
       <c r="O169" s="2" t="n"/>
       <c r="P169" s="2" t="n"/>
+      <c r="Q169" s="2" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n"/>
@@ -6161,6 +6348,7 @@
       <c r="N170" s="2" t="n"/>
       <c r="O170" s="2" t="n"/>
       <c r="P170" s="2" t="n"/>
+      <c r="Q170" s="2" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n"/>
@@ -6193,6 +6381,7 @@
       <c r="N171" s="2" t="n"/>
       <c r="O171" s="2" t="n"/>
       <c r="P171" s="2" t="n"/>
+      <c r="Q171" s="2" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n"/>
@@ -6225,6 +6414,7 @@
       <c r="N172" s="2" t="n"/>
       <c r="O172" s="2" t="n"/>
       <c r="P172" s="2" t="n"/>
+      <c r="Q172" s="2" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n"/>
@@ -6257,6 +6447,7 @@
       <c r="N173" s="2" t="n"/>
       <c r="O173" s="2" t="n"/>
       <c r="P173" s="2" t="n"/>
+      <c r="Q173" s="2" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n"/>
@@ -6289,6 +6480,7 @@
       <c r="N174" s="2" t="n"/>
       <c r="O174" s="2" t="n"/>
       <c r="P174" s="2" t="n"/>
+      <c r="Q174" s="2" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n"/>
@@ -6321,6 +6513,7 @@
       <c r="N175" s="2" t="n"/>
       <c r="O175" s="2" t="n"/>
       <c r="P175" s="2" t="n"/>
+      <c r="Q175" s="2" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n"/>
@@ -6353,6 +6546,7 @@
       <c r="N176" s="2" t="n"/>
       <c r="O176" s="2" t="n"/>
       <c r="P176" s="2" t="n"/>
+      <c r="Q176" s="2" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n"/>
@@ -6385,6 +6579,7 @@
       <c r="N177" s="2" t="n"/>
       <c r="O177" s="2" t="n"/>
       <c r="P177" s="2" t="n"/>
+      <c r="Q177" s="2" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n"/>
@@ -6417,6 +6612,7 @@
       <c r="N178" s="2" t="n"/>
       <c r="O178" s="2" t="n"/>
       <c r="P178" s="2" t="n"/>
+      <c r="Q178" s="2" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n"/>
@@ -6449,6 +6645,7 @@
       <c r="N179" s="2" t="n"/>
       <c r="O179" s="2" t="n"/>
       <c r="P179" s="2" t="n"/>
+      <c r="Q179" s="2" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n"/>
@@ -6481,6 +6678,7 @@
       <c r="N180" s="2" t="n"/>
       <c r="O180" s="2" t="n"/>
       <c r="P180" s="2" t="n"/>
+      <c r="Q180" s="2" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n"/>
@@ -6513,6 +6711,7 @@
       <c r="N181" s="2" t="n"/>
       <c r="O181" s="2" t="n"/>
       <c r="P181" s="2" t="n"/>
+      <c r="Q181" s="2" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n"/>
@@ -6545,6 +6744,7 @@
       <c r="N182" s="2" t="n"/>
       <c r="O182" s="2" t="n"/>
       <c r="P182" s="2" t="n"/>
+      <c r="Q182" s="2" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n"/>
@@ -6577,6 +6777,7 @@
       <c r="N183" s="2" t="n"/>
       <c r="O183" s="2" t="n"/>
       <c r="P183" s="2" t="n"/>
+      <c r="Q183" s="2" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n"/>
@@ -6609,6 +6810,7 @@
       <c r="N184" s="2" t="n"/>
       <c r="O184" s="2" t="n"/>
       <c r="P184" s="2" t="n"/>
+      <c r="Q184" s="2" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n"/>
@@ -6641,6 +6843,7 @@
       <c r="N185" s="2" t="n"/>
       <c r="O185" s="2" t="n"/>
       <c r="P185" s="2" t="n"/>
+      <c r="Q185" s="2" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n"/>
@@ -6673,6 +6876,7 @@
       <c r="N186" s="2" t="n"/>
       <c r="O186" s="2" t="n"/>
       <c r="P186" s="2" t="n"/>
+      <c r="Q186" s="2" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n"/>
@@ -6705,6 +6909,7 @@
       <c r="N187" s="2" t="n"/>
       <c r="O187" s="2" t="n"/>
       <c r="P187" s="2" t="n"/>
+      <c r="Q187" s="2" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n"/>
@@ -6737,6 +6942,7 @@
       <c r="N188" s="2" t="n"/>
       <c r="O188" s="2" t="n"/>
       <c r="P188" s="2" t="n"/>
+      <c r="Q188" s="2" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n"/>
@@ -6769,6 +6975,7 @@
       <c r="N189" s="2" t="n"/>
       <c r="O189" s="2" t="n"/>
       <c r="P189" s="2" t="n"/>
+      <c r="Q189" s="2" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n"/>
@@ -6801,6 +7008,7 @@
       <c r="N190" s="2" t="n"/>
       <c r="O190" s="2" t="n"/>
       <c r="P190" s="2" t="n"/>
+      <c r="Q190" s="2" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n"/>
@@ -6833,6 +7041,7 @@
       <c r="N191" s="2" t="n"/>
       <c r="O191" s="2" t="n"/>
       <c r="P191" s="2" t="n"/>
+      <c r="Q191" s="2" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n"/>
@@ -6865,6 +7074,7 @@
       <c r="N192" s="2" t="n"/>
       <c r="O192" s="2" t="n"/>
       <c r="P192" s="2" t="n"/>
+      <c r="Q192" s="2" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n"/>
@@ -6897,6 +7107,7 @@
       <c r="N193" s="2" t="n"/>
       <c r="O193" s="2" t="n"/>
       <c r="P193" s="2" t="n"/>
+      <c r="Q193" s="2" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n"/>
@@ -6929,6 +7140,7 @@
       <c r="N194" s="2" t="n"/>
       <c r="O194" s="2" t="n"/>
       <c r="P194" s="2" t="n"/>
+      <c r="Q194" s="2" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n"/>
@@ -6961,6 +7173,7 @@
       <c r="N195" s="2" t="n"/>
       <c r="O195" s="2" t="n"/>
       <c r="P195" s="2" t="n"/>
+      <c r="Q195" s="2" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n"/>
@@ -6993,6 +7206,7 @@
       <c r="N196" s="2" t="n"/>
       <c r="O196" s="2" t="n"/>
       <c r="P196" s="2" t="n"/>
+      <c r="Q196" s="2" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n"/>
@@ -7025,6 +7239,7 @@
       <c r="N197" s="2" t="n"/>
       <c r="O197" s="2" t="n"/>
       <c r="P197" s="2" t="n"/>
+      <c r="Q197" s="2" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n"/>
@@ -7057,6 +7272,7 @@
       <c r="N198" s="2" t="n"/>
       <c r="O198" s="2" t="n"/>
       <c r="P198" s="2" t="n"/>
+      <c r="Q198" s="2" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n"/>
@@ -7089,6 +7305,7 @@
       <c r="N199" s="2" t="n"/>
       <c r="O199" s="2" t="n"/>
       <c r="P199" s="2" t="n"/>
+      <c r="Q199" s="2" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n"/>
@@ -7121,6 +7338,7 @@
       <c r="N200" s="2" t="n"/>
       <c r="O200" s="2" t="n"/>
       <c r="P200" s="2" t="n"/>
+      <c r="Q200" s="2" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n"/>
@@ -7153,6 +7371,7 @@
       <c r="N201" s="2" t="n"/>
       <c r="O201" s="2" t="n"/>
       <c r="P201" s="2" t="n"/>
+      <c r="Q201" s="2" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="n"/>
@@ -7185,6 +7404,7 @@
       <c r="N202" s="2" t="n"/>
       <c r="O202" s="2" t="n"/>
       <c r="P202" s="2" t="n"/>
+      <c r="Q202" s="2" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="n"/>
@@ -7217,6 +7437,7 @@
       <c r="N203" s="2" t="n"/>
       <c r="O203" s="2" t="n"/>
       <c r="P203" s="2" t="n"/>
+      <c r="Q203" s="2" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n"/>
@@ -7249,6 +7470,7 @@
       <c r="N204" s="2" t="n"/>
       <c r="O204" s="2" t="n"/>
       <c r="P204" s="2" t="n"/>
+      <c r="Q204" s="2" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n"/>
@@ -7281,6 +7503,7 @@
       <c r="N205" s="2" t="n"/>
       <c r="O205" s="2" t="n"/>
       <c r="P205" s="2" t="n"/>
+      <c r="Q205" s="2" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="n"/>
@@ -7313,6 +7536,7 @@
       <c r="N206" s="2" t="n"/>
       <c r="O206" s="2" t="n"/>
       <c r="P206" s="2" t="n"/>
+      <c r="Q206" s="2" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="n"/>
@@ -7345,6 +7569,7 @@
       <c r="N207" s="2" t="n"/>
       <c r="O207" s="2" t="n"/>
       <c r="P207" s="2" t="n"/>
+      <c r="Q207" s="2" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n"/>
@@ -7377,6 +7602,7 @@
       <c r="N208" s="2" t="n"/>
       <c r="O208" s="2" t="n"/>
       <c r="P208" s="2" t="n"/>
+      <c r="Q208" s="2" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="n"/>
@@ -7409,6 +7635,7 @@
       <c r="N209" s="2" t="n"/>
       <c r="O209" s="2" t="n"/>
       <c r="P209" s="2" t="n"/>
+      <c r="Q209" s="2" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n"/>
@@ -7441,6 +7668,7 @@
       <c r="N210" s="2" t="n"/>
       <c r="O210" s="2" t="n"/>
       <c r="P210" s="2" t="n"/>
+      <c r="Q210" s="2" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="n"/>
@@ -7473,6 +7701,7 @@
       <c r="N211" s="2" t="n"/>
       <c r="O211" s="2" t="n"/>
       <c r="P211" s="2" t="n"/>
+      <c r="Q211" s="2" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="n"/>
@@ -7505,6 +7734,7 @@
       <c r="N212" s="2" t="n"/>
       <c r="O212" s="2" t="n"/>
       <c r="P212" s="2" t="n"/>
+      <c r="Q212" s="2" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="n"/>
@@ -7537,6 +7767,7 @@
       <c r="N213" s="2" t="n"/>
       <c r="O213" s="2" t="n"/>
       <c r="P213" s="2" t="n"/>
+      <c r="Q213" s="2" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="2" t="n"/>
@@ -7569,6 +7800,7 @@
       <c r="N214" s="2" t="n"/>
       <c r="O214" s="2" t="n"/>
       <c r="P214" s="2" t="n"/>
+      <c r="Q214" s="2" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="2" t="n"/>
@@ -7601,6 +7833,7 @@
       <c r="N215" s="2" t="n"/>
       <c r="O215" s="2" t="n"/>
       <c r="P215" s="2" t="n"/>
+      <c r="Q215" s="2" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="2" t="n"/>
@@ -7633,6 +7866,7 @@
       <c r="N216" s="2" t="n"/>
       <c r="O216" s="2" t="n"/>
       <c r="P216" s="2" t="n"/>
+      <c r="Q216" s="2" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="2" t="n"/>
@@ -7665,6 +7899,7 @@
       <c r="N217" s="2" t="n"/>
       <c r="O217" s="2" t="n"/>
       <c r="P217" s="2" t="n"/>
+      <c r="Q217" s="2" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="n"/>
@@ -7697,6 +7932,7 @@
       <c r="N218" s="2" t="n"/>
       <c r="O218" s="2" t="n"/>
       <c r="P218" s="2" t="n"/>
+      <c r="Q218" s="2" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="2" t="n"/>
@@ -7729,6 +7965,7 @@
       <c r="N219" s="2" t="n"/>
       <c r="O219" s="2" t="n"/>
       <c r="P219" s="2" t="n"/>
+      <c r="Q219" s="2" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="n"/>
@@ -7761,6 +7998,7 @@
       <c r="N220" s="2" t="n"/>
       <c r="O220" s="2" t="n"/>
       <c r="P220" s="2" t="n"/>
+      <c r="Q220" s="2" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="2" t="n"/>
@@ -7793,6 +8031,7 @@
       <c r="N221" s="2" t="n"/>
       <c r="O221" s="2" t="n"/>
       <c r="P221" s="2" t="n"/>
+      <c r="Q221" s="2" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="2" t="n"/>
@@ -7825,6 +8064,7 @@
       <c r="N222" s="2" t="n"/>
       <c r="O222" s="2" t="n"/>
       <c r="P222" s="2" t="n"/>
+      <c r="Q222" s="2" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="n"/>
@@ -7857,6 +8097,7 @@
       <c r="N223" s="2" t="n"/>
       <c r="O223" s="2" t="n"/>
       <c r="P223" s="2" t="n"/>
+      <c r="Q223" s="2" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="2" t="n"/>
@@ -7889,6 +8130,7 @@
       <c r="N224" s="2" t="n"/>
       <c r="O224" s="2" t="n"/>
       <c r="P224" s="2" t="n"/>
+      <c r="Q224" s="2" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="2" t="n"/>
@@ -7921,6 +8163,7 @@
       <c r="N225" s="2" t="n"/>
       <c r="O225" s="2" t="n"/>
       <c r="P225" s="2" t="n"/>
+      <c r="Q225" s="2" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="n"/>
@@ -7953,6 +8196,7 @@
       <c r="N226" s="2" t="n"/>
       <c r="O226" s="2" t="n"/>
       <c r="P226" s="2" t="n"/>
+      <c r="Q226" s="2" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="2" t="n"/>
@@ -7985,6 +8229,7 @@
       <c r="N227" s="2" t="n"/>
       <c r="O227" s="2" t="n"/>
       <c r="P227" s="2" t="n"/>
+      <c r="Q227" s="2" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="2" t="n"/>
@@ -8017,6 +8262,7 @@
       <c r="N228" s="2" t="n"/>
       <c r="O228" s="2" t="n"/>
       <c r="P228" s="2" t="n"/>
+      <c r="Q228" s="2" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="n"/>
@@ -8049,6 +8295,7 @@
       <c r="N229" s="2" t="n"/>
       <c r="O229" s="2" t="n"/>
       <c r="P229" s="2" t="n"/>
+      <c r="Q229" s="2" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="2" t="n"/>
@@ -8081,6 +8328,7 @@
       <c r="N230" s="2" t="n"/>
       <c r="O230" s="2" t="n"/>
       <c r="P230" s="2" t="n"/>
+      <c r="Q230" s="2" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="2" t="n"/>
@@ -8113,6 +8361,7 @@
       <c r="N231" s="2" t="n"/>
       <c r="O231" s="2" t="n"/>
       <c r="P231" s="2" t="n"/>
+      <c r="Q231" s="2" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="2" t="n"/>
@@ -8145,6 +8394,7 @@
       <c r="N232" s="2" t="n"/>
       <c r="O232" s="2" t="n"/>
       <c r="P232" s="2" t="n"/>
+      <c r="Q232" s="2" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="2" t="n"/>
@@ -8177,6 +8427,7 @@
       <c r="N233" s="2" t="n"/>
       <c r="O233" s="2" t="n"/>
       <c r="P233" s="2" t="n"/>
+      <c r="Q233" s="2" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="2" t="n"/>
@@ -8209,6 +8460,7 @@
       <c r="N234" s="2" t="n"/>
       <c r="O234" s="2" t="n"/>
       <c r="P234" s="2" t="n"/>
+      <c r="Q234" s="2" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="2" t="n"/>
@@ -8241,6 +8493,7 @@
       <c r="N235" s="2" t="n"/>
       <c r="O235" s="2" t="n"/>
       <c r="P235" s="2" t="n"/>
+      <c r="Q235" s="2" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="2" t="n"/>
@@ -8273,6 +8526,7 @@
       <c r="N236" s="2" t="n"/>
       <c r="O236" s="2" t="n"/>
       <c r="P236" s="2" t="n"/>
+      <c r="Q236" s="2" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="n"/>
@@ -8305,6 +8559,7 @@
       <c r="N237" s="2" t="n"/>
       <c r="O237" s="2" t="n"/>
       <c r="P237" s="2" t="n"/>
+      <c r="Q237" s="2" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="n"/>
@@ -8337,6 +8592,7 @@
       <c r="N238" s="2" t="n"/>
       <c r="O238" s="2" t="n"/>
       <c r="P238" s="2" t="n"/>
+      <c r="Q238" s="2" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="2" t="n"/>
@@ -8369,6 +8625,7 @@
       <c r="N239" s="2" t="n"/>
       <c r="O239" s="2" t="n"/>
       <c r="P239" s="2" t="n"/>
+      <c r="Q239" s="2" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="2" t="n"/>
@@ -8401,6 +8658,7 @@
       <c r="N240" s="2" t="n"/>
       <c r="O240" s="2" t="n"/>
       <c r="P240" s="2" t="n"/>
+      <c r="Q240" s="2" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="2" t="n"/>
@@ -8433,6 +8691,7 @@
       <c r="N241" s="2" t="n"/>
       <c r="O241" s="2" t="n"/>
       <c r="P241" s="2" t="n"/>
+      <c r="Q241" s="2" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="2" t="n"/>
@@ -8465,6 +8724,7 @@
       <c r="N242" s="2" t="n"/>
       <c r="O242" s="2" t="n"/>
       <c r="P242" s="2" t="n"/>
+      <c r="Q242" s="2" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="2" t="n"/>
@@ -8497,6 +8757,7 @@
       <c r="N243" s="2" t="n"/>
       <c r="O243" s="2" t="n"/>
       <c r="P243" s="2" t="n"/>
+      <c r="Q243" s="2" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="n"/>
@@ -8529,6 +8790,7 @@
       <c r="N244" s="2" t="n"/>
       <c r="O244" s="2" t="n"/>
       <c r="P244" s="2" t="n"/>
+      <c r="Q244" s="2" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="n"/>
@@ -8561,6 +8823,7 @@
       <c r="N245" s="2" t="n"/>
       <c r="O245" s="2" t="n"/>
       <c r="P245" s="2" t="n"/>
+      <c r="Q245" s="2" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="2" t="n"/>
@@ -8593,6 +8856,7 @@
       <c r="N246" s="2" t="n"/>
       <c r="O246" s="2" t="n"/>
       <c r="P246" s="2" t="n"/>
+      <c r="Q246" s="2" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="2" t="n"/>
@@ -8625,6 +8889,7 @@
       <c r="N247" s="2" t="n"/>
       <c r="O247" s="2" t="n"/>
       <c r="P247" s="2" t="n"/>
+      <c r="Q247" s="2" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="2" t="n"/>
@@ -8657,6 +8922,7 @@
       <c r="N248" s="2" t="n"/>
       <c r="O248" s="2" t="n"/>
       <c r="P248" s="2" t="n"/>
+      <c r="Q248" s="2" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="2" t="n"/>
@@ -8689,6 +8955,7 @@
       <c r="N249" s="2" t="n"/>
       <c r="O249" s="2" t="n"/>
       <c r="P249" s="2" t="n"/>
+      <c r="Q249" s="2" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="2" t="n"/>
@@ -8721,6 +8988,7 @@
       <c r="N250" s="2" t="n"/>
       <c r="O250" s="2" t="n"/>
       <c r="P250" s="2" t="n"/>
+      <c r="Q250" s="2" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="2" t="n"/>
@@ -8753,6 +9021,7 @@
       <c r="N251" s="2" t="n"/>
       <c r="O251" s="2" t="n"/>
       <c r="P251" s="2" t="n"/>
+      <c r="Q251" s="2" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="2" t="n"/>
@@ -8785,6 +9054,7 @@
       <c r="N252" s="2" t="n"/>
       <c r="O252" s="2" t="n"/>
       <c r="P252" s="2" t="n"/>
+      <c r="Q252" s="2" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="2" t="n"/>
@@ -8817,6 +9087,7 @@
       <c r="N253" s="2" t="n"/>
       <c r="O253" s="2" t="n"/>
       <c r="P253" s="2" t="n"/>
+      <c r="Q253" s="2" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="2" t="n"/>
@@ -8849,6 +9120,7 @@
       <c r="N254" s="2" t="n"/>
       <c r="O254" s="2" t="n"/>
       <c r="P254" s="2" t="n"/>
+      <c r="Q254" s="2" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="2" t="n"/>
@@ -8881,6 +9153,7 @@
       <c r="N255" s="2" t="n"/>
       <c r="O255" s="2" t="n"/>
       <c r="P255" s="2" t="n"/>
+      <c r="Q255" s="2" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="2" t="n"/>
@@ -8913,6 +9186,7 @@
       <c r="N256" s="2" t="n"/>
       <c r="O256" s="2" t="n"/>
       <c r="P256" s="2" t="n"/>
+      <c r="Q256" s="2" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="2" t="n"/>
@@ -8945,6 +9219,7 @@
       <c r="N257" s="2" t="n"/>
       <c r="O257" s="2" t="n"/>
       <c r="P257" s="2" t="n"/>
+      <c r="Q257" s="2" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="2" t="n"/>
@@ -8977,6 +9252,7 @@
       <c r="N258" s="2" t="n"/>
       <c r="O258" s="2" t="n"/>
       <c r="P258" s="2" t="n"/>
+      <c r="Q258" s="2" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="2" t="n"/>
@@ -9009,6 +9285,7 @@
       <c r="N259" s="2" t="n"/>
       <c r="O259" s="2" t="n"/>
       <c r="P259" s="2" t="n"/>
+      <c r="Q259" s="2" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="2" t="n"/>
@@ -9041,6 +9318,7 @@
       <c r="N260" s="2" t="n"/>
       <c r="O260" s="2" t="n"/>
       <c r="P260" s="2" t="n"/>
+      <c r="Q260" s="2" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="2" t="n"/>
@@ -9073,6 +9351,7 @@
       <c r="N261" s="2" t="n"/>
       <c r="O261" s="2" t="n"/>
       <c r="P261" s="2" t="n"/>
+      <c r="Q261" s="2" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="2" t="n"/>
@@ -9105,6 +9384,7 @@
       <c r="N262" s="2" t="n"/>
       <c r="O262" s="2" t="n"/>
       <c r="P262" s="2" t="n"/>
+      <c r="Q262" s="2" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="2" t="n"/>
@@ -9137,6 +9417,7 @@
       <c r="N263" s="2" t="n"/>
       <c r="O263" s="2" t="n"/>
       <c r="P263" s="2" t="n"/>
+      <c r="Q263" s="2" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="2" t="n"/>
@@ -9169,6 +9450,7 @@
       <c r="N264" s="2" t="n"/>
       <c r="O264" s="2" t="n"/>
       <c r="P264" s="2" t="n"/>
+      <c r="Q264" s="2" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="2" t="n"/>
@@ -9201,6 +9483,7 @@
       <c r="N265" s="2" t="n"/>
       <c r="O265" s="2" t="n"/>
       <c r="P265" s="2" t="n"/>
+      <c r="Q265" s="2" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="2" t="n"/>
@@ -9233,6 +9516,7 @@
       <c r="N266" s="2" t="n"/>
       <c r="O266" s="2" t="n"/>
       <c r="P266" s="2" t="n"/>
+      <c r="Q266" s="2" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="2" t="n"/>
@@ -9265,6 +9549,7 @@
       <c r="N267" s="2" t="n"/>
       <c r="O267" s="2" t="n"/>
       <c r="P267" s="2" t="n"/>
+      <c r="Q267" s="2" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="2" t="n"/>
@@ -9297,6 +9582,7 @@
       <c r="N268" s="2" t="n"/>
       <c r="O268" s="2" t="n"/>
       <c r="P268" s="2" t="n"/>
+      <c r="Q268" s="2" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="2" t="n"/>
@@ -9329,6 +9615,7 @@
       <c r="N269" s="2" t="n"/>
       <c r="O269" s="2" t="n"/>
       <c r="P269" s="2" t="n"/>
+      <c r="Q269" s="2" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="2" t="n"/>
@@ -9361,6 +9648,7 @@
       <c r="N270" s="2" t="n"/>
       <c r="O270" s="2" t="n"/>
       <c r="P270" s="2" t="n"/>
+      <c r="Q270" s="2" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="2" t="n"/>
@@ -9393,6 +9681,7 @@
       <c r="N271" s="2" t="n"/>
       <c r="O271" s="2" t="n"/>
       <c r="P271" s="2" t="n"/>
+      <c r="Q271" s="2" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="2" t="n"/>
@@ -9425,6 +9714,7 @@
       <c r="N272" s="2" t="n"/>
       <c r="O272" s="2" t="n"/>
       <c r="P272" s="2" t="n"/>
+      <c r="Q272" s="2" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="2" t="n"/>
@@ -9457,6 +9747,7 @@
       <c r="N273" s="2" t="n"/>
       <c r="O273" s="2" t="n"/>
       <c r="P273" s="2" t="n"/>
+      <c r="Q273" s="2" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="2" t="n"/>
@@ -9489,6 +9780,7 @@
       <c r="N274" s="2" t="n"/>
       <c r="O274" s="2" t="n"/>
       <c r="P274" s="2" t="n"/>
+      <c r="Q274" s="2" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="2" t="n"/>
@@ -9521,6 +9813,7 @@
       <c r="N275" s="2" t="n"/>
       <c r="O275" s="2" t="n"/>
       <c r="P275" s="2" t="n"/>
+      <c r="Q275" s="2" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="2" t="n"/>
@@ -9553,6 +9846,7 @@
       <c r="N276" s="2" t="n"/>
       <c r="O276" s="2" t="n"/>
       <c r="P276" s="2" t="n"/>
+      <c r="Q276" s="2" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="2" t="n"/>
@@ -9585,6 +9879,7 @@
       <c r="N277" s="2" t="n"/>
       <c r="O277" s="2" t="n"/>
       <c r="P277" s="2" t="n"/>
+      <c r="Q277" s="2" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="2" t="n"/>
@@ -9617,6 +9912,7 @@
       <c r="N278" s="2" t="n"/>
       <c r="O278" s="2" t="n"/>
       <c r="P278" s="2" t="n"/>
+      <c r="Q278" s="2" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="2" t="n"/>
@@ -9649,6 +9945,7 @@
       <c r="N279" s="2" t="n"/>
       <c r="O279" s="2" t="n"/>
       <c r="P279" s="2" t="n"/>
+      <c r="Q279" s="2" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="2" t="n"/>
@@ -9681,6 +9978,7 @@
       <c r="N280" s="2" t="n"/>
       <c r="O280" s="2" t="n"/>
       <c r="P280" s="2" t="n"/>
+      <c r="Q280" s="2" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="2" t="n"/>
@@ -9713,6 +10011,7 @@
       <c r="N281" s="2" t="n"/>
       <c r="O281" s="2" t="n"/>
       <c r="P281" s="2" t="n"/>
+      <c r="Q281" s="2" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="2" t="n"/>
@@ -9745,6 +10044,7 @@
       <c r="N282" s="2" t="n"/>
       <c r="O282" s="2" t="n"/>
       <c r="P282" s="2" t="n"/>
+      <c r="Q282" s="2" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="2" t="n"/>
@@ -9777,6 +10077,7 @@
       <c r="N283" s="2" t="n"/>
       <c r="O283" s="2" t="n"/>
       <c r="P283" s="2" t="n"/>
+      <c r="Q283" s="2" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="2" t="n"/>
@@ -9809,6 +10110,7 @@
       <c r="N284" s="2" t="n"/>
       <c r="O284" s="2" t="n"/>
       <c r="P284" s="2" t="n"/>
+      <c r="Q284" s="2" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="2" t="n"/>
@@ -9841,6 +10143,7 @@
       <c r="N285" s="2" t="n"/>
       <c r="O285" s="2" t="n"/>
       <c r="P285" s="2" t="n"/>
+      <c r="Q285" s="2" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="2" t="n"/>
@@ -9873,6 +10176,7 @@
       <c r="N286" s="2" t="n"/>
       <c r="O286" s="2" t="n"/>
       <c r="P286" s="2" t="n"/>
+      <c r="Q286" s="2" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="2" t="n"/>
@@ -9905,6 +10209,7 @@
       <c r="N287" s="2" t="n"/>
       <c r="O287" s="2" t="n"/>
       <c r="P287" s="2" t="n"/>
+      <c r="Q287" s="2" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="2" t="n"/>
@@ -9937,6 +10242,7 @@
       <c r="N288" s="2" t="n"/>
       <c r="O288" s="2" t="n"/>
       <c r="P288" s="2" t="n"/>
+      <c r="Q288" s="2" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="2" t="n"/>
@@ -9969,6 +10275,7 @@
       <c r="N289" s="2" t="n"/>
       <c r="O289" s="2" t="n"/>
       <c r="P289" s="2" t="n"/>
+      <c r="Q289" s="2" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="2" t="n"/>
@@ -10001,6 +10308,7 @@
       <c r="N290" s="2" t="n"/>
       <c r="O290" s="2" t="n"/>
       <c r="P290" s="2" t="n"/>
+      <c r="Q290" s="2" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="2" t="n"/>
@@ -10033,6 +10341,7 @@
       <c r="N291" s="2" t="n"/>
       <c r="O291" s="2" t="n"/>
       <c r="P291" s="2" t="n"/>
+      <c r="Q291" s="2" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="2" t="n"/>
@@ -10065,6 +10374,7 @@
       <c r="N292" s="2" t="n"/>
       <c r="O292" s="2" t="n"/>
       <c r="P292" s="2" t="n"/>
+      <c r="Q292" s="2" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="2" t="n"/>
@@ -10097,6 +10407,7 @@
       <c r="N293" s="2" t="n"/>
       <c r="O293" s="2" t="n"/>
       <c r="P293" s="2" t="n"/>
+      <c r="Q293" s="2" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="2" t="n"/>
@@ -10129,6 +10440,7 @@
       <c r="N294" s="2" t="n"/>
       <c r="O294" s="2" t="n"/>
       <c r="P294" s="2" t="n"/>
+      <c r="Q294" s="2" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="2" t="n"/>
@@ -10161,6 +10473,7 @@
       <c r="N295" s="2" t="n"/>
       <c r="O295" s="2" t="n"/>
       <c r="P295" s="2" t="n"/>
+      <c r="Q295" s="2" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="2" t="n"/>
@@ -10193,6 +10506,7 @@
       <c r="N296" s="2" t="n"/>
       <c r="O296" s="2" t="n"/>
       <c r="P296" s="2" t="n"/>
+      <c r="Q296" s="2" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="2" t="n"/>
@@ -10225,6 +10539,7 @@
       <c r="N297" s="2" t="n"/>
       <c r="O297" s="2" t="n"/>
       <c r="P297" s="2" t="n"/>
+      <c r="Q297" s="2" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="2" t="n"/>
@@ -10257,6 +10572,7 @@
       <c r="N298" s="2" t="n"/>
       <c r="O298" s="2" t="n"/>
       <c r="P298" s="2" t="n"/>
+      <c r="Q298" s="2" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="2" t="n"/>
@@ -10289,6 +10605,7 @@
       <c r="N299" s="2" t="n"/>
       <c r="O299" s="2" t="n"/>
       <c r="P299" s="2" t="n"/>
+      <c r="Q299" s="2" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="2" t="n"/>
@@ -10321,6 +10638,7 @@
       <c r="N300" s="2" t="n"/>
       <c r="O300" s="2" t="n"/>
       <c r="P300" s="2" t="n"/>
+      <c r="Q300" s="2" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="2" t="n"/>
@@ -10353,6 +10671,7 @@
       <c r="N301" s="2" t="n"/>
       <c r="O301" s="2" t="n"/>
       <c r="P301" s="2" t="n"/>
+      <c r="Q301" s="2" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="2" t="n"/>
@@ -10385,6 +10704,7 @@
       <c r="N302" s="2" t="n"/>
       <c r="O302" s="2" t="n"/>
       <c r="P302" s="2" t="n"/>
+      <c r="Q302" s="2" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="2" t="n"/>
@@ -10417,6 +10737,7 @@
       <c r="N303" s="2" t="n"/>
       <c r="O303" s="2" t="n"/>
       <c r="P303" s="2" t="n"/>
+      <c r="Q303" s="2" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="2" t="n"/>
@@ -10449,6 +10770,7 @@
       <c r="N304" s="2" t="n"/>
       <c r="O304" s="2" t="n"/>
       <c r="P304" s="2" t="n"/>
+      <c r="Q304" s="2" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="2" t="n"/>
@@ -10481,6 +10803,7 @@
       <c r="N305" s="2" t="n"/>
       <c r="O305" s="2" t="n"/>
       <c r="P305" s="2" t="n"/>
+      <c r="Q305" s="2" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="2" t="n"/>
@@ -10513,6 +10836,7 @@
       <c r="N306" s="2" t="n"/>
       <c r="O306" s="2" t="n"/>
       <c r="P306" s="2" t="n"/>
+      <c r="Q306" s="2" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="2" t="n"/>
@@ -10545,6 +10869,7 @@
       <c r="N307" s="2" t="n"/>
       <c r="O307" s="2" t="n"/>
       <c r="P307" s="2" t="n"/>
+      <c r="Q307" s="2" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="2" t="n"/>
@@ -10577,6 +10902,7 @@
       <c r="N308" s="2" t="n"/>
       <c r="O308" s="2" t="n"/>
       <c r="P308" s="2" t="n"/>
+      <c r="Q308" s="2" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="2" t="n"/>
@@ -10609,6 +10935,7 @@
       <c r="N309" s="2" t="n"/>
       <c r="O309" s="2" t="n"/>
       <c r="P309" s="2" t="n"/>
+      <c r="Q309" s="2" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="2" t="n"/>
@@ -10641,6 +10968,7 @@
       <c r="N310" s="2" t="n"/>
       <c r="O310" s="2" t="n"/>
       <c r="P310" s="2" t="n"/>
+      <c r="Q310" s="2" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="2" t="n"/>
@@ -10673,6 +11001,7 @@
       <c r="N311" s="2" t="n"/>
       <c r="O311" s="2" t="n"/>
       <c r="P311" s="2" t="n"/>
+      <c r="Q311" s="2" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="2" t="n"/>
@@ -10705,6 +11034,7 @@
       <c r="N312" s="2" t="n"/>
       <c r="O312" s="2" t="n"/>
       <c r="P312" s="2" t="n"/>
+      <c r="Q312" s="2" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="2" t="n"/>
@@ -10737,6 +11067,7 @@
       <c r="N313" s="2" t="n"/>
       <c r="O313" s="2" t="n"/>
       <c r="P313" s="2" t="n"/>
+      <c r="Q313" s="2" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="2" t="n"/>
@@ -10769,6 +11100,7 @@
       <c r="N314" s="2" t="n"/>
       <c r="O314" s="2" t="n"/>
       <c r="P314" s="2" t="n"/>
+      <c r="Q314" s="2" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="2" t="n"/>
@@ -10801,6 +11133,7 @@
       <c r="N315" s="2" t="n"/>
       <c r="O315" s="2" t="n"/>
       <c r="P315" s="2" t="n"/>
+      <c r="Q315" s="2" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="2" t="n"/>
@@ -10833,6 +11166,7 @@
       <c r="N316" s="2" t="n"/>
       <c r="O316" s="2" t="n"/>
       <c r="P316" s="2" t="n"/>
+      <c r="Q316" s="2" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="2" t="n"/>
@@ -10865,6 +11199,7 @@
       <c r="N317" s="2" t="n"/>
       <c r="O317" s="2" t="n"/>
       <c r="P317" s="2" t="n"/>
+      <c r="Q317" s="2" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="2" t="n"/>
@@ -10897,6 +11232,7 @@
       <c r="N318" s="2" t="n"/>
       <c r="O318" s="2" t="n"/>
       <c r="P318" s="2" t="n"/>
+      <c r="Q318" s="2" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="2" t="n"/>
@@ -10929,6 +11265,7 @@
       <c r="N319" s="2" t="n"/>
       <c r="O319" s="2" t="n"/>
       <c r="P319" s="2" t="n"/>
+      <c r="Q319" s="2" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="2" t="n"/>
@@ -10961,6 +11298,7 @@
       <c r="N320" s="2" t="n"/>
       <c r="O320" s="2" t="n"/>
       <c r="P320" s="2" t="n"/>
+      <c r="Q320" s="2" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="2" t="n"/>
@@ -10993,6 +11331,7 @@
       <c r="N321" s="2" t="n"/>
       <c r="O321" s="2" t="n"/>
       <c r="P321" s="2" t="n"/>
+      <c r="Q321" s="2" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="2" t="n"/>
@@ -11025,6 +11364,7 @@
       <c r="N322" s="2" t="n"/>
       <c r="O322" s="2" t="n"/>
       <c r="P322" s="2" t="n"/>
+      <c r="Q322" s="2" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="2" t="n"/>
@@ -11057,6 +11397,7 @@
       <c r="N323" s="2" t="n"/>
       <c r="O323" s="2" t="n"/>
       <c r="P323" s="2" t="n"/>
+      <c r="Q323" s="2" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="2" t="n"/>
@@ -11089,6 +11430,7 @@
       <c r="N324" s="2" t="n"/>
       <c r="O324" s="2" t="n"/>
       <c r="P324" s="2" t="n"/>
+      <c r="Q324" s="2" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="2" t="n"/>
@@ -11121,6 +11463,7 @@
       <c r="N325" s="2" t="n"/>
       <c r="O325" s="2" t="n"/>
       <c r="P325" s="2" t="n"/>
+      <c r="Q325" s="2" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="2" t="n"/>
@@ -11153,6 +11496,7 @@
       <c r="N326" s="2" t="n"/>
       <c r="O326" s="2" t="n"/>
       <c r="P326" s="2" t="n"/>
+      <c r="Q326" s="2" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="2" t="n"/>
@@ -11185,6 +11529,7 @@
       <c r="N327" s="2" t="n"/>
       <c r="O327" s="2" t="n"/>
       <c r="P327" s="2" t="n"/>
+      <c r="Q327" s="2" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="2" t="n"/>
@@ -11217,6 +11562,7 @@
       <c r="N328" s="2" t="n"/>
       <c r="O328" s="2" t="n"/>
       <c r="P328" s="2" t="n"/>
+      <c r="Q328" s="2" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="2" t="n"/>
@@ -11249,6 +11595,7 @@
       <c r="N329" s="2" t="n"/>
       <c r="O329" s="2" t="n"/>
       <c r="P329" s="2" t="n"/>
+      <c r="Q329" s="2" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="2" t="n"/>
@@ -11281,6 +11628,7 @@
       <c r="N330" s="2" t="n"/>
       <c r="O330" s="2" t="n"/>
       <c r="P330" s="2" t="n"/>
+      <c r="Q330" s="2" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="2" t="n"/>
@@ -11313,6 +11661,7 @@
       <c r="N331" s="2" t="n"/>
       <c r="O331" s="2" t="n"/>
       <c r="P331" s="2" t="n"/>
+      <c r="Q331" s="2" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="2" t="n"/>
@@ -11345,6 +11694,7 @@
       <c r="N332" s="2" t="n"/>
       <c r="O332" s="2" t="n"/>
       <c r="P332" s="2" t="n"/>
+      <c r="Q332" s="2" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="2" t="n"/>
@@ -11377,6 +11727,7 @@
       <c r="N333" s="2" t="n"/>
       <c r="O333" s="2" t="n"/>
       <c r="P333" s="2" t="n"/>
+      <c r="Q333" s="2" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="2" t="n"/>
@@ -11409,6 +11760,7 @@
       <c r="N334" s="2" t="n"/>
       <c r="O334" s="2" t="n"/>
       <c r="P334" s="2" t="n"/>
+      <c r="Q334" s="2" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="2" t="n"/>
@@ -11441,6 +11793,7 @@
       <c r="N335" s="2" t="n"/>
       <c r="O335" s="2" t="n"/>
       <c r="P335" s="2" t="n"/>
+      <c r="Q335" s="2" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="2" t="n"/>
@@ -11473,6 +11826,7 @@
       <c r="N336" s="2" t="n"/>
       <c r="O336" s="2" t="n"/>
       <c r="P336" s="2" t="n"/>
+      <c r="Q336" s="2" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="2" t="n"/>
@@ -11505,6 +11859,7 @@
       <c r="N337" s="2" t="n"/>
       <c r="O337" s="2" t="n"/>
       <c r="P337" s="2" t="n"/>
+      <c r="Q337" s="2" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="2" t="n"/>
@@ -11537,6 +11892,7 @@
       <c r="N338" s="2" t="n"/>
       <c r="O338" s="2" t="n"/>
       <c r="P338" s="2" t="n"/>
+      <c r="Q338" s="2" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="2" t="n"/>
@@ -11569,6 +11925,7 @@
       <c r="N339" s="2" t="n"/>
       <c r="O339" s="2" t="n"/>
       <c r="P339" s="2" t="n"/>
+      <c r="Q339" s="2" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="2" t="n"/>
@@ -11601,6 +11958,7 @@
       <c r="N340" s="2" t="n"/>
       <c r="O340" s="2" t="n"/>
       <c r="P340" s="2" t="n"/>
+      <c r="Q340" s="2" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="2" t="n"/>
@@ -11633,6 +11991,7 @@
       <c r="N341" s="2" t="n"/>
       <c r="O341" s="2" t="n"/>
       <c r="P341" s="2" t="n"/>
+      <c r="Q341" s="2" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="2" t="n"/>
@@ -11665,6 +12024,7 @@
       <c r="N342" s="2" t="n"/>
       <c r="O342" s="2" t="n"/>
       <c r="P342" s="2" t="n"/>
+      <c r="Q342" s="2" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="2" t="n"/>
@@ -11697,6 +12057,7 @@
       <c r="N343" s="2" t="n"/>
       <c r="O343" s="2" t="n"/>
       <c r="P343" s="2" t="n"/>
+      <c r="Q343" s="2" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="2" t="n"/>
@@ -11729,6 +12090,7 @@
       <c r="N344" s="2" t="n"/>
       <c r="O344" s="2" t="n"/>
       <c r="P344" s="2" t="n"/>
+      <c r="Q344" s="2" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="2" t="n"/>
@@ -11761,6 +12123,7 @@
       <c r="N345" s="2" t="n"/>
       <c r="O345" s="2" t="n"/>
       <c r="P345" s="2" t="n"/>
+      <c r="Q345" s="2" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="2" t="n"/>
@@ -11793,6 +12156,7 @@
       <c r="N346" s="2" t="n"/>
       <c r="O346" s="2" t="n"/>
       <c r="P346" s="2" t="n"/>
+      <c r="Q346" s="2" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="2" t="n"/>
@@ -11825,6 +12189,7 @@
       <c r="N347" s="2" t="n"/>
       <c r="O347" s="2" t="n"/>
       <c r="P347" s="2" t="n"/>
+      <c r="Q347" s="2" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="2" t="n"/>
@@ -11857,6 +12222,7 @@
       <c r="N348" s="2" t="n"/>
       <c r="O348" s="2" t="n"/>
       <c r="P348" s="2" t="n"/>
+      <c r="Q348" s="2" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="2" t="n"/>
@@ -11889,6 +12255,7 @@
       <c r="N349" s="2" t="n"/>
       <c r="O349" s="2" t="n"/>
       <c r="P349" s="2" t="n"/>
+      <c r="Q349" s="2" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="2" t="n"/>
@@ -11921,6 +12288,7 @@
       <c r="N350" s="2" t="n"/>
       <c r="O350" s="2" t="n"/>
       <c r="P350" s="2" t="n"/>
+      <c r="Q350" s="2" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="2" t="n"/>
@@ -11953,6 +12321,7 @@
       <c r="N351" s="2" t="n"/>
       <c r="O351" s="2" t="n"/>
       <c r="P351" s="2" t="n"/>
+      <c r="Q351" s="2" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="2" t="n"/>
@@ -11985,6 +12354,7 @@
       <c r="N352" s="2" t="n"/>
       <c r="O352" s="2" t="n"/>
       <c r="P352" s="2" t="n"/>
+      <c r="Q352" s="2" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="2" t="n"/>
@@ -12017,6 +12387,7 @@
       <c r="N353" s="2" t="n"/>
       <c r="O353" s="2" t="n"/>
       <c r="P353" s="2" t="n"/>
+      <c r="Q353" s="2" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="2" t="n"/>
@@ -12049,6 +12420,7 @@
       <c r="N354" s="2" t="n"/>
       <c r="O354" s="2" t="n"/>
       <c r="P354" s="2" t="n"/>
+      <c r="Q354" s="2" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="2" t="n"/>
@@ -12081,6 +12453,7 @@
       <c r="N355" s="2" t="n"/>
       <c r="O355" s="2" t="n"/>
       <c r="P355" s="2" t="n"/>
+      <c r="Q355" s="2" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="2" t="n"/>
@@ -12113,6 +12486,7 @@
       <c r="N356" s="2" t="n"/>
       <c r="O356" s="2" t="n"/>
       <c r="P356" s="2" t="n"/>
+      <c r="Q356" s="2" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="2" t="n"/>
@@ -12145,6 +12519,7 @@
       <c r="N357" s="2" t="n"/>
       <c r="O357" s="2" t="n"/>
       <c r="P357" s="2" t="n"/>
+      <c r="Q357" s="2" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="2" t="n"/>
@@ -12177,6 +12552,7 @@
       <c r="N358" s="2" t="n"/>
       <c r="O358" s="2" t="n"/>
       <c r="P358" s="2" t="n"/>
+      <c r="Q358" s="2" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="2" t="n"/>
@@ -12209,6 +12585,7 @@
       <c r="N359" s="2" t="n"/>
       <c r="O359" s="2" t="n"/>
       <c r="P359" s="2" t="n"/>
+      <c r="Q359" s="2" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="2" t="n"/>
@@ -12241,6 +12618,7 @@
       <c r="N360" s="2" t="n"/>
       <c r="O360" s="2" t="n"/>
       <c r="P360" s="2" t="n"/>
+      <c r="Q360" s="2" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="2" t="n"/>
@@ -12273,6 +12651,7 @@
       <c r="N361" s="2" t="n"/>
       <c r="O361" s="2" t="n"/>
       <c r="P361" s="2" t="n"/>
+      <c r="Q361" s="2" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="2" t="n"/>
@@ -12305,6 +12684,7 @@
       <c r="N362" s="2" t="n"/>
       <c r="O362" s="2" t="n"/>
       <c r="P362" s="2" t="n"/>
+      <c r="Q362" s="2" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="2" t="n"/>
@@ -12337,6 +12717,7 @@
       <c r="N363" s="2" t="n"/>
       <c r="O363" s="2" t="n"/>
       <c r="P363" s="2" t="n"/>
+      <c r="Q363" s="2" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="2" t="n"/>
@@ -12369,6 +12750,7 @@
       <c r="N364" s="2" t="n"/>
       <c r="O364" s="2" t="n"/>
       <c r="P364" s="2" t="n"/>
+      <c r="Q364" s="2" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="2" t="n"/>
@@ -12401,6 +12783,7 @@
       <c r="N365" s="2" t="n"/>
       <c r="O365" s="2" t="n"/>
       <c r="P365" s="2" t="n"/>
+      <c r="Q365" s="2" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="2" t="n"/>
@@ -12433,6 +12816,7 @@
       <c r="N366" s="2" t="n"/>
       <c r="O366" s="2" t="n"/>
       <c r="P366" s="2" t="n"/>
+      <c r="Q366" s="2" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="2" t="n"/>
@@ -12465,6 +12849,7 @@
       <c r="N367" s="2" t="n"/>
       <c r="O367" s="2" t="n"/>
       <c r="P367" s="2" t="n"/>
+      <c r="Q367" s="2" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="2" t="n"/>
@@ -12497,6 +12882,7 @@
       <c r="N368" s="2" t="n"/>
       <c r="O368" s="2" t="n"/>
       <c r="P368" s="2" t="n"/>
+      <c r="Q368" s="2" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="2" t="n"/>
@@ -12529,6 +12915,7 @@
       <c r="N369" s="2" t="n"/>
       <c r="O369" s="2" t="n"/>
       <c r="P369" s="2" t="n"/>
+      <c r="Q369" s="2" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="2" t="n"/>
@@ -12561,6 +12948,7 @@
       <c r="N370" s="2" t="n"/>
       <c r="O370" s="2" t="n"/>
       <c r="P370" s="2" t="n"/>
+      <c r="Q370" s="2" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="2" t="n"/>
@@ -12593,6 +12981,7 @@
       <c r="N371" s="2" t="n"/>
       <c r="O371" s="2" t="n"/>
       <c r="P371" s="2" t="n"/>
+      <c r="Q371" s="2" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="2" t="n"/>
@@ -12625,6 +13014,7 @@
       <c r="N372" s="2" t="n"/>
       <c r="O372" s="2" t="n"/>
       <c r="P372" s="2" t="n"/>
+      <c r="Q372" s="2" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="2" t="n"/>
@@ -12657,6 +13047,7 @@
       <c r="N373" s="2" t="n"/>
       <c r="O373" s="2" t="n"/>
       <c r="P373" s="2" t="n"/>
+      <c r="Q373" s="2" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="2" t="n"/>
@@ -12689,6 +13080,7 @@
       <c r="N374" s="2" t="n"/>
       <c r="O374" s="2" t="n"/>
       <c r="P374" s="2" t="n"/>
+      <c r="Q374" s="2" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="2" t="n"/>
@@ -12721,6 +13113,7 @@
       <c r="N375" s="2" t="n"/>
       <c r="O375" s="2" t="n"/>
       <c r="P375" s="2" t="n"/>
+      <c r="Q375" s="2" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="2" t="n"/>
@@ -12753,6 +13146,7 @@
       <c r="N376" s="2" t="n"/>
       <c r="O376" s="2" t="n"/>
       <c r="P376" s="2" t="n"/>
+      <c r="Q376" s="2" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="2" t="n"/>
@@ -12785,6 +13179,7 @@
       <c r="N377" s="2" t="n"/>
       <c r="O377" s="2" t="n"/>
       <c r="P377" s="2" t="n"/>
+      <c r="Q377" s="2" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="2" t="n"/>
@@ -12817,6 +13212,7 @@
       <c r="N378" s="2" t="n"/>
       <c r="O378" s="2" t="n"/>
       <c r="P378" s="2" t="n"/>
+      <c r="Q378" s="2" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="2" t="n"/>
@@ -12849,6 +13245,7 @@
       <c r="N379" s="2" t="n"/>
       <c r="O379" s="2" t="n"/>
       <c r="P379" s="2" t="n"/>
+      <c r="Q379" s="2" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="2" t="n"/>
@@ -12881,6 +13278,7 @@
       <c r="N380" s="2" t="n"/>
       <c r="O380" s="2" t="n"/>
       <c r="P380" s="2" t="n"/>
+      <c r="Q380" s="2" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="2" t="n"/>
@@ -12913,6 +13311,7 @@
       <c r="N381" s="2" t="n"/>
       <c r="O381" s="2" t="n"/>
       <c r="P381" s="2" t="n"/>
+      <c r="Q381" s="2" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="2" t="n"/>
@@ -12945,6 +13344,7 @@
       <c r="N382" s="2" t="n"/>
       <c r="O382" s="2" t="n"/>
       <c r="P382" s="2" t="n"/>
+      <c r="Q382" s="2" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="2" t="n"/>
@@ -12977,6 +13377,7 @@
       <c r="N383" s="2" t="n"/>
       <c r="O383" s="2" t="n"/>
       <c r="P383" s="2" t="n"/>
+      <c r="Q383" s="2" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="2" t="n"/>
@@ -13009,6 +13410,7 @@
       <c r="N384" s="2" t="n"/>
       <c r="O384" s="2" t="n"/>
       <c r="P384" s="2" t="n"/>
+      <c r="Q384" s="2" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="2" t="n"/>
@@ -13041,6 +13443,7 @@
       <c r="N385" s="2" t="n"/>
       <c r="O385" s="2" t="n"/>
       <c r="P385" s="2" t="n"/>
+      <c r="Q385" s="2" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="2" t="n"/>
@@ -13073,6 +13476,7 @@
       <c r="N386" s="2" t="n"/>
       <c r="O386" s="2" t="n"/>
       <c r="P386" s="2" t="n"/>
+      <c r="Q386" s="2" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="2" t="n"/>
@@ -13105,6 +13509,7 @@
       <c r="N387" s="2" t="n"/>
       <c r="O387" s="2" t="n"/>
       <c r="P387" s="2" t="n"/>
+      <c r="Q387" s="2" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="2" t="n"/>
@@ -13137,6 +13542,7 @@
       <c r="N388" s="2" t="n"/>
       <c r="O388" s="2" t="n"/>
       <c r="P388" s="2" t="n"/>
+      <c r="Q388" s="2" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="2" t="n"/>
@@ -13169,6 +13575,7 @@
       <c r="N389" s="2" t="n"/>
       <c r="O389" s="2" t="n"/>
       <c r="P389" s="2" t="n"/>
+      <c r="Q389" s="2" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="2" t="n"/>
@@ -13201,6 +13608,7 @@
       <c r="N390" s="2" t="n"/>
       <c r="O390" s="2" t="n"/>
       <c r="P390" s="2" t="n"/>
+      <c r="Q390" s="2" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="2" t="n"/>
@@ -13233,6 +13641,7 @@
       <c r="N391" s="2" t="n"/>
       <c r="O391" s="2" t="n"/>
       <c r="P391" s="2" t="n"/>
+      <c r="Q391" s="2" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="2" t="n"/>
@@ -13265,6 +13674,7 @@
       <c r="N392" s="2" t="n"/>
       <c r="O392" s="2" t="n"/>
       <c r="P392" s="2" t="n"/>
+      <c r="Q392" s="2" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="2" t="n"/>
@@ -13297,6 +13707,7 @@
       <c r="N393" s="2" t="n"/>
       <c r="O393" s="2" t="n"/>
       <c r="P393" s="2" t="n"/>
+      <c r="Q393" s="2" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="2" t="n"/>
@@ -13329,6 +13740,7 @@
       <c r="N394" s="2" t="n"/>
       <c r="O394" s="2" t="n"/>
       <c r="P394" s="2" t="n"/>
+      <c r="Q394" s="2" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="2" t="n"/>
@@ -13361,6 +13773,7 @@
       <c r="N395" s="2" t="n"/>
       <c r="O395" s="2" t="n"/>
       <c r="P395" s="2" t="n"/>
+      <c r="Q395" s="2" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="2" t="n"/>
@@ -13393,6 +13806,7 @@
       <c r="N396" s="2" t="n"/>
       <c r="O396" s="2" t="n"/>
       <c r="P396" s="2" t="n"/>
+      <c r="Q396" s="2" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="2" t="n"/>
@@ -13425,6 +13839,7 @@
       <c r="N397" s="2" t="n"/>
       <c r="O397" s="2" t="n"/>
       <c r="P397" s="2" t="n"/>
+      <c r="Q397" s="2" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="2" t="n"/>
@@ -13457,6 +13872,7 @@
       <c r="N398" s="2" t="n"/>
       <c r="O398" s="2" t="n"/>
       <c r="P398" s="2" t="n"/>
+      <c r="Q398" s="2" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="2" t="n"/>
@@ -13489,6 +13905,7 @@
       <c r="N399" s="2" t="n"/>
       <c r="O399" s="2" t="n"/>
       <c r="P399" s="2" t="n"/>
+      <c r="Q399" s="2" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="2" t="n"/>
@@ -13521,6 +13938,7 @@
       <c r="N400" s="2" t="n"/>
       <c r="O400" s="2" t="n"/>
       <c r="P400" s="2" t="n"/>
+      <c r="Q400" s="2" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="2" t="n"/>
@@ -13553,6 +13971,7 @@
       <c r="N401" s="2" t="n"/>
       <c r="O401" s="2" t="n"/>
       <c r="P401" s="2" t="n"/>
+      <c r="Q401" s="2" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="2" t="n"/>
@@ -13585,6 +14004,7 @@
       <c r="N402" s="2" t="n"/>
       <c r="O402" s="2" t="n"/>
       <c r="P402" s="2" t="n"/>
+      <c r="Q402" s="2" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="2" t="n"/>
@@ -13617,6 +14037,7 @@
       <c r="N403" s="2" t="n"/>
       <c r="O403" s="2" t="n"/>
       <c r="P403" s="2" t="n"/>
+      <c r="Q403" s="2" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="2" t="n"/>
@@ -13649,6 +14070,7 @@
       <c r="N404" s="2" t="n"/>
       <c r="O404" s="2" t="n"/>
       <c r="P404" s="2" t="n"/>
+      <c r="Q404" s="2" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="2" t="n"/>
@@ -13681,6 +14103,7 @@
       <c r="N405" s="2" t="n"/>
       <c r="O405" s="2" t="n"/>
       <c r="P405" s="2" t="n"/>
+      <c r="Q405" s="2" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="2" t="n"/>
@@ -13713,6 +14136,7 @@
       <c r="N406" s="2" t="n"/>
       <c r="O406" s="2" t="n"/>
       <c r="P406" s="2" t="n"/>
+      <c r="Q406" s="2" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="2" t="n"/>
@@ -13745,6 +14169,7 @@
       <c r="N407" s="2" t="n"/>
       <c r="O407" s="2" t="n"/>
       <c r="P407" s="2" t="n"/>
+      <c r="Q407" s="2" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="2" t="n"/>
@@ -13777,6 +14202,7 @@
       <c r="N408" s="2" t="n"/>
       <c r="O408" s="2" t="n"/>
       <c r="P408" s="2" t="n"/>
+      <c r="Q408" s="2" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="2" t="n"/>
@@ -13809,6 +14235,7 @@
       <c r="N409" s="2" t="n"/>
       <c r="O409" s="2" t="n"/>
       <c r="P409" s="2" t="n"/>
+      <c r="Q409" s="2" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="2" t="n"/>
@@ -13841,6 +14268,7 @@
       <c r="N410" s="2" t="n"/>
       <c r="O410" s="2" t="n"/>
       <c r="P410" s="2" t="n"/>
+      <c r="Q410" s="2" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="2" t="n"/>
@@ -13873,6 +14301,7 @@
       <c r="N411" s="2" t="n"/>
       <c r="O411" s="2" t="n"/>
       <c r="P411" s="2" t="n"/>
+      <c r="Q411" s="2" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="2" t="n"/>
@@ -13905,6 +14334,7 @@
       <c r="N412" s="2" t="n"/>
       <c r="O412" s="2" t="n"/>
       <c r="P412" s="2" t="n"/>
+      <c r="Q412" s="2" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="2" t="n"/>
@@ -13937,6 +14367,7 @@
       <c r="N413" s="2" t="n"/>
       <c r="O413" s="2" t="n"/>
       <c r="P413" s="2" t="n"/>
+      <c r="Q413" s="2" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="2" t="n"/>
@@ -13969,6 +14400,7 @@
       <c r="N414" s="2" t="n"/>
       <c r="O414" s="2" t="n"/>
       <c r="P414" s="2" t="n"/>
+      <c r="Q414" s="2" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="2" t="n"/>
@@ -14001,6 +14433,7 @@
       <c r="N415" s="2" t="n"/>
       <c r="O415" s="2" t="n"/>
       <c r="P415" s="2" t="n"/>
+      <c r="Q415" s="2" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="2" t="n"/>
@@ -14033,6 +14466,7 @@
       <c r="N416" s="2" t="n"/>
       <c r="O416" s="2" t="n"/>
       <c r="P416" s="2" t="n"/>
+      <c r="Q416" s="2" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="2" t="n"/>
@@ -14065,6 +14499,7 @@
       <c r="N417" s="2" t="n"/>
       <c r="O417" s="2" t="n"/>
       <c r="P417" s="2" t="n"/>
+      <c r="Q417" s="2" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="2" t="n"/>
@@ -14097,6 +14532,7 @@
       <c r="N418" s="2" t="n"/>
       <c r="O418" s="2" t="n"/>
       <c r="P418" s="2" t="n"/>
+      <c r="Q418" s="2" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="2" t="n"/>
@@ -14129,6 +14565,7 @@
       <c r="N419" s="2" t="n"/>
       <c r="O419" s="2" t="n"/>
       <c r="P419" s="2" t="n"/>
+      <c r="Q419" s="2" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="2" t="n"/>
@@ -14161,6 +14598,7 @@
       <c r="N420" s="2" t="n"/>
       <c r="O420" s="2" t="n"/>
       <c r="P420" s="2" t="n"/>
+      <c r="Q420" s="2" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="2" t="n"/>
@@ -14193,6 +14631,7 @@
       <c r="N421" s="2" t="n"/>
       <c r="O421" s="2" t="n"/>
       <c r="P421" s="2" t="n"/>
+      <c r="Q421" s="2" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="2" t="n"/>
@@ -14225,6 +14664,7 @@
       <c r="N422" s="2" t="n"/>
       <c r="O422" s="2" t="n"/>
       <c r="P422" s="2" t="n"/>
+      <c r="Q422" s="2" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="2" t="n"/>
@@ -14257,6 +14697,7 @@
       <c r="N423" s="2" t="n"/>
       <c r="O423" s="2" t="n"/>
       <c r="P423" s="2" t="n"/>
+      <c r="Q423" s="2" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="2" t="n"/>
@@ -14289,6 +14730,7 @@
       <c r="N424" s="2" t="n"/>
       <c r="O424" s="2" t="n"/>
       <c r="P424" s="2" t="n"/>
+      <c r="Q424" s="2" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="2" t="n"/>
@@ -14321,6 +14763,7 @@
       <c r="N425" s="2" t="n"/>
       <c r="O425" s="2" t="n"/>
       <c r="P425" s="2" t="n"/>
+      <c r="Q425" s="2" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="2" t="n"/>
@@ -14353,6 +14796,7 @@
       <c r="N426" s="2" t="n"/>
       <c r="O426" s="2" t="n"/>
       <c r="P426" s="2" t="n"/>
+      <c r="Q426" s="2" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="2" t="n"/>
@@ -14385,6 +14829,7 @@
       <c r="N427" s="2" t="n"/>
       <c r="O427" s="2" t="n"/>
       <c r="P427" s="2" t="n"/>
+      <c r="Q427" s="2" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="2" t="n"/>
@@ -14417,6 +14862,7 @@
       <c r="N428" s="2" t="n"/>
       <c r="O428" s="2" t="n"/>
       <c r="P428" s="2" t="n"/>
+      <c r="Q428" s="2" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="2" t="n"/>
@@ -14449,6 +14895,7 @@
       <c r="N429" s="2" t="n"/>
       <c r="O429" s="2" t="n"/>
       <c r="P429" s="2" t="n"/>
+      <c r="Q429" s="2" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="2" t="n"/>
@@ -14481,6 +14928,7 @@
       <c r="N430" s="2" t="n"/>
       <c r="O430" s="2" t="n"/>
       <c r="P430" s="2" t="n"/>
+      <c r="Q430" s="2" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="2" t="n"/>
@@ -14513,6 +14961,7 @@
       <c r="N431" s="2" t="n"/>
       <c r="O431" s="2" t="n"/>
       <c r="P431" s="2" t="n"/>
+      <c r="Q431" s="2" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="2" t="n"/>
@@ -14545,6 +14994,7 @@
       <c r="N432" s="2" t="n"/>
       <c r="O432" s="2" t="n"/>
       <c r="P432" s="2" t="n"/>
+      <c r="Q432" s="2" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="2" t="n"/>
@@ -14577,6 +15027,7 @@
       <c r="N433" s="2" t="n"/>
       <c r="O433" s="2" t="n"/>
       <c r="P433" s="2" t="n"/>
+      <c r="Q433" s="2" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="2" t="n"/>
@@ -14609,6 +15060,7 @@
       <c r="N434" s="2" t="n"/>
       <c r="O434" s="2" t="n"/>
       <c r="P434" s="2" t="n"/>
+      <c r="Q434" s="2" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="2" t="n"/>
@@ -14641,6 +15093,7 @@
       <c r="N435" s="2" t="n"/>
       <c r="O435" s="2" t="n"/>
       <c r="P435" s="2" t="n"/>
+      <c r="Q435" s="2" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="2" t="n"/>
@@ -14673,6 +15126,7 @@
       <c r="N436" s="2" t="n"/>
       <c r="O436" s="2" t="n"/>
       <c r="P436" s="2" t="n"/>
+      <c r="Q436" s="2" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="2" t="n"/>
@@ -14705,6 +15159,7 @@
       <c r="N437" s="2" t="n"/>
       <c r="O437" s="2" t="n"/>
       <c r="P437" s="2" t="n"/>
+      <c r="Q437" s="2" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="2" t="n"/>
@@ -14737,6 +15192,7 @@
       <c r="N438" s="2" t="n"/>
       <c r="O438" s="2" t="n"/>
       <c r="P438" s="2" t="n"/>
+      <c r="Q438" s="2" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="2" t="n"/>
@@ -14769,6 +15225,7 @@
       <c r="N439" s="2" t="n"/>
       <c r="O439" s="2" t="n"/>
       <c r="P439" s="2" t="n"/>
+      <c r="Q439" s="2" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="2" t="n"/>
@@ -14801,6 +15258,7 @@
       <c r="N440" s="2" t="n"/>
       <c r="O440" s="2" t="n"/>
       <c r="P440" s="2" t="n"/>
+      <c r="Q440" s="2" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="2" t="n"/>
@@ -14833,6 +15291,7 @@
       <c r="N441" s="2" t="n"/>
       <c r="O441" s="2" t="n"/>
       <c r="P441" s="2" t="n"/>
+      <c r="Q441" s="2" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="2" t="n"/>
@@ -14865,6 +15324,7 @@
       <c r="N442" s="2" t="n"/>
       <c r="O442" s="2" t="n"/>
       <c r="P442" s="2" t="n"/>
+      <c r="Q442" s="2" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="2" t="n"/>
@@ -14897,6 +15357,7 @@
       <c r="N443" s="2" t="n"/>
       <c r="O443" s="2" t="n"/>
       <c r="P443" s="2" t="n"/>
+      <c r="Q443" s="2" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="2" t="n"/>
@@ -14929,6 +15390,7 @@
       <c r="N444" s="2" t="n"/>
       <c r="O444" s="2" t="n"/>
       <c r="P444" s="2" t="n"/>
+      <c r="Q444" s="2" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="2" t="n"/>
@@ -14961,6 +15423,7 @@
       <c r="N445" s="2" t="n"/>
       <c r="O445" s="2" t="n"/>
       <c r="P445" s="2" t="n"/>
+      <c r="Q445" s="2" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="2" t="n"/>
@@ -14993,6 +15456,7 @@
       <c r="N446" s="2" t="n"/>
       <c r="O446" s="2" t="n"/>
       <c r="P446" s="2" t="n"/>
+      <c r="Q446" s="2" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="2" t="n"/>
@@ -15025,6 +15489,7 @@
       <c r="N447" s="2" t="n"/>
       <c r="O447" s="2" t="n"/>
       <c r="P447" s="2" t="n"/>
+      <c r="Q447" s="2" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="2" t="n"/>
@@ -15057,6 +15522,7 @@
       <c r="N448" s="2" t="n"/>
       <c r="O448" s="2" t="n"/>
       <c r="P448" s="2" t="n"/>
+      <c r="Q448" s="2" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="2" t="n"/>
@@ -15089,6 +15555,7 @@
       <c r="N449" s="2" t="n"/>
       <c r="O449" s="2" t="n"/>
       <c r="P449" s="2" t="n"/>
+      <c r="Q449" s="2" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="2" t="n"/>
@@ -15121,6 +15588,7 @@
       <c r="N450" s="2" t="n"/>
       <c r="O450" s="2" t="n"/>
       <c r="P450" s="2" t="n"/>
+      <c r="Q450" s="2" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="2" t="n"/>
@@ -15153,6 +15621,7 @@
       <c r="N451" s="2" t="n"/>
       <c r="O451" s="2" t="n"/>
       <c r="P451" s="2" t="n"/>
+      <c r="Q451" s="2" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="2" t="n"/>
@@ -15185,6 +15654,7 @@
       <c r="N452" s="2" t="n"/>
       <c r="O452" s="2" t="n"/>
       <c r="P452" s="2" t="n"/>
+      <c r="Q452" s="2" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="2" t="n"/>
@@ -15217,6 +15687,7 @@
       <c r="N453" s="2" t="n"/>
       <c r="O453" s="2" t="n"/>
       <c r="P453" s="2" t="n"/>
+      <c r="Q453" s="2" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="2" t="n"/>
@@ -15249,6 +15720,7 @@
       <c r="N454" s="2" t="n"/>
       <c r="O454" s="2" t="n"/>
       <c r="P454" s="2" t="n"/>
+      <c r="Q454" s="2" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="2" t="n"/>
@@ -15281,6 +15753,7 @@
       <c r="N455" s="2" t="n"/>
       <c r="O455" s="2" t="n"/>
       <c r="P455" s="2" t="n"/>
+      <c r="Q455" s="2" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="2" t="n"/>
@@ -15313,6 +15786,7 @@
       <c r="N456" s="2" t="n"/>
       <c r="O456" s="2" t="n"/>
       <c r="P456" s="2" t="n"/>
+      <c r="Q456" s="2" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="2" t="n"/>
@@ -15345,6 +15819,7 @@
       <c r="N457" s="2" t="n"/>
       <c r="O457" s="2" t="n"/>
       <c r="P457" s="2" t="n"/>
+      <c r="Q457" s="2" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="2" t="n"/>
@@ -15377,6 +15852,7 @@
       <c r="N458" s="2" t="n"/>
       <c r="O458" s="2" t="n"/>
       <c r="P458" s="2" t="n"/>
+      <c r="Q458" s="2" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="2" t="n"/>
@@ -15409,6 +15885,7 @@
       <c r="N459" s="2" t="n"/>
       <c r="O459" s="2" t="n"/>
       <c r="P459" s="2" t="n"/>
+      <c r="Q459" s="2" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="2" t="n"/>
@@ -15441,6 +15918,7 @@
       <c r="N460" s="2" t="n"/>
       <c r="O460" s="2" t="n"/>
       <c r="P460" s="2" t="n"/>
+      <c r="Q460" s="2" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="2" t="n"/>
@@ -15473,6 +15951,7 @@
       <c r="N461" s="2" t="n"/>
       <c r="O461" s="2" t="n"/>
       <c r="P461" s="2" t="n"/>
+      <c r="Q461" s="2" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="2" t="n"/>
@@ -15505,6 +15984,7 @@
       <c r="N462" s="2" t="n"/>
       <c r="O462" s="2" t="n"/>
       <c r="P462" s="2" t="n"/>
+      <c r="Q462" s="2" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="2" t="n"/>
@@ -15537,6 +16017,7 @@
       <c r="N463" s="2" t="n"/>
       <c r="O463" s="2" t="n"/>
       <c r="P463" s="2" t="n"/>
+      <c r="Q463" s="2" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="2" t="n"/>
@@ -15569,6 +16050,7 @@
       <c r="N464" s="2" t="n"/>
       <c r="O464" s="2" t="n"/>
       <c r="P464" s="2" t="n"/>
+      <c r="Q464" s="2" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="2" t="n"/>
@@ -15601,6 +16083,7 @@
       <c r="N465" s="2" t="n"/>
       <c r="O465" s="2" t="n"/>
       <c r="P465" s="2" t="n"/>
+      <c r="Q465" s="2" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="2" t="n"/>
@@ -15633,6 +16116,7 @@
       <c r="N466" s="2" t="n"/>
       <c r="O466" s="2" t="n"/>
       <c r="P466" s="2" t="n"/>
+      <c r="Q466" s="2" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="2" t="n"/>
@@ -15665,6 +16149,7 @@
       <c r="N467" s="2" t="n"/>
       <c r="O467" s="2" t="n"/>
       <c r="P467" s="2" t="n"/>
+      <c r="Q467" s="2" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="2" t="n"/>
@@ -15697,6 +16182,7 @@
       <c r="N468" s="2" t="n"/>
       <c r="O468" s="2" t="n"/>
       <c r="P468" s="2" t="n"/>
+      <c r="Q468" s="2" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="2" t="n"/>
@@ -15729,6 +16215,7 @@
       <c r="N469" s="2" t="n"/>
       <c r="O469" s="2" t="n"/>
       <c r="P469" s="2" t="n"/>
+      <c r="Q469" s="2" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="2" t="n"/>
@@ -15761,6 +16248,7 @@
       <c r="N470" s="2" t="n"/>
       <c r="O470" s="2" t="n"/>
       <c r="P470" s="2" t="n"/>
+      <c r="Q470" s="2" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="2" t="n"/>
@@ -15793,6 +16281,7 @@
       <c r="N471" s="2" t="n"/>
       <c r="O471" s="2" t="n"/>
       <c r="P471" s="2" t="n"/>
+      <c r="Q471" s="2" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="2" t="n"/>
@@ -15825,6 +16314,7 @@
       <c r="N472" s="2" t="n"/>
       <c r="O472" s="2" t="n"/>
       <c r="P472" s="2" t="n"/>
+      <c r="Q472" s="2" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="2" t="n"/>
@@ -15857,6 +16347,7 @@
       <c r="N473" s="2" t="n"/>
       <c r="O473" s="2" t="n"/>
       <c r="P473" s="2" t="n"/>
+      <c r="Q473" s="2" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="2" t="n"/>
@@ -15889,6 +16380,7 @@
       <c r="N474" s="2" t="n"/>
       <c r="O474" s="2" t="n"/>
       <c r="P474" s="2" t="n"/>
+      <c r="Q474" s="2" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="2" t="n"/>
@@ -15921,6 +16413,7 @@
       <c r="N475" s="2" t="n"/>
       <c r="O475" s="2" t="n"/>
       <c r="P475" s="2" t="n"/>
+      <c r="Q475" s="2" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="2" t="n"/>
@@ -15953,6 +16446,7 @@
       <c r="N476" s="2" t="n"/>
       <c r="O476" s="2" t="n"/>
       <c r="P476" s="2" t="n"/>
+      <c r="Q476" s="2" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="2" t="n"/>
@@ -15985,6 +16479,7 @@
       <c r="N477" s="2" t="n"/>
       <c r="O477" s="2" t="n"/>
       <c r="P477" s="2" t="n"/>
+      <c r="Q477" s="2" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="2" t="n"/>
@@ -16017,6 +16512,7 @@
       <c r="N478" s="2" t="n"/>
       <c r="O478" s="2" t="n"/>
       <c r="P478" s="2" t="n"/>
+      <c r="Q478" s="2" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="2" t="n"/>
@@ -16049,6 +16545,7 @@
       <c r="N479" s="2" t="n"/>
       <c r="O479" s="2" t="n"/>
       <c r="P479" s="2" t="n"/>
+      <c r="Q479" s="2" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="2" t="n"/>
@@ -16081,6 +16578,7 @@
       <c r="N480" s="2" t="n"/>
       <c r="O480" s="2" t="n"/>
       <c r="P480" s="2" t="n"/>
+      <c r="Q480" s="2" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="2" t="n"/>
@@ -16113,6 +16611,7 @@
       <c r="N481" s="2" t="n"/>
       <c r="O481" s="2" t="n"/>
       <c r="P481" s="2" t="n"/>
+      <c r="Q481" s="2" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="2" t="n"/>
@@ -16145,6 +16644,7 @@
       <c r="N482" s="2" t="n"/>
       <c r="O482" s="2" t="n"/>
       <c r="P482" s="2" t="n"/>
+      <c r="Q482" s="2" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="2" t="n"/>
@@ -16177,6 +16677,7 @@
       <c r="N483" s="2" t="n"/>
       <c r="O483" s="2" t="n"/>
       <c r="P483" s="2" t="n"/>
+      <c r="Q483" s="2" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="2" t="n"/>
@@ -16209,6 +16710,7 @@
       <c r="N484" s="2" t="n"/>
       <c r="O484" s="2" t="n"/>
       <c r="P484" s="2" t="n"/>
+      <c r="Q484" s="2" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="2" t="n"/>
@@ -16241,6 +16743,7 @@
       <c r="N485" s="2" t="n"/>
       <c r="O485" s="2" t="n"/>
       <c r="P485" s="2" t="n"/>
+      <c r="Q485" s="2" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="2" t="n"/>
@@ -16273,6 +16776,7 @@
       <c r="N486" s="2" t="n"/>
       <c r="O486" s="2" t="n"/>
       <c r="P486" s="2" t="n"/>
+      <c r="Q486" s="2" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="2" t="n"/>
@@ -16305,6 +16809,7 @@
       <c r="N487" s="2" t="n"/>
       <c r="O487" s="2" t="n"/>
       <c r="P487" s="2" t="n"/>
+      <c r="Q487" s="2" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="2" t="n"/>
@@ -16337,6 +16842,7 @@
       <c r="N488" s="2" t="n"/>
       <c r="O488" s="2" t="n"/>
       <c r="P488" s="2" t="n"/>
+      <c r="Q488" s="2" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="2" t="n"/>
@@ -16369,6 +16875,7 @@
       <c r="N489" s="2" t="n"/>
       <c r="O489" s="2" t="n"/>
       <c r="P489" s="2" t="n"/>
+      <c r="Q489" s="2" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="2" t="n"/>
@@ -16401,6 +16908,7 @@
       <c r="N490" s="2" t="n"/>
       <c r="O490" s="2" t="n"/>
       <c r="P490" s="2" t="n"/>
+      <c r="Q490" s="2" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="2" t="n"/>
@@ -16433,6 +16941,7 @@
       <c r="N491" s="2" t="n"/>
       <c r="O491" s="2" t="n"/>
       <c r="P491" s="2" t="n"/>
+      <c r="Q491" s="2" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="2" t="n"/>
@@ -16465,6 +16974,7 @@
       <c r="N492" s="2" t="n"/>
       <c r="O492" s="2" t="n"/>
       <c r="P492" s="2" t="n"/>
+      <c r="Q492" s="2" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="2" t="n"/>
@@ -16497,6 +17007,7 @@
       <c r="N493" s="2" t="n"/>
       <c r="O493" s="2" t="n"/>
       <c r="P493" s="2" t="n"/>
+      <c r="Q493" s="2" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="2" t="n"/>
@@ -16529,6 +17040,7 @@
       <c r="N494" s="2" t="n"/>
       <c r="O494" s="2" t="n"/>
       <c r="P494" s="2" t="n"/>
+      <c r="Q494" s="2" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="2" t="n"/>
@@ -16561,6 +17073,7 @@
       <c r="N495" s="2" t="n"/>
       <c r="O495" s="2" t="n"/>
       <c r="P495" s="2" t="n"/>
+      <c r="Q495" s="2" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="2" t="n"/>
@@ -16593,6 +17106,7 @@
       <c r="N496" s="2" t="n"/>
       <c r="O496" s="2" t="n"/>
       <c r="P496" s="2" t="n"/>
+      <c r="Q496" s="2" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="2" t="n"/>
@@ -16625,6 +17139,7 @@
       <c r="N497" s="2" t="n"/>
       <c r="O497" s="2" t="n"/>
       <c r="P497" s="2" t="n"/>
+      <c r="Q497" s="2" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="2" t="n"/>
@@ -16657,6 +17172,7 @@
       <c r="N498" s="2" t="n"/>
       <c r="O498" s="2" t="n"/>
       <c r="P498" s="2" t="n"/>
+      <c r="Q498" s="2" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="2" t="n"/>
@@ -16689,6 +17205,7 @@
       <c r="N499" s="2" t="n"/>
       <c r="O499" s="2" t="n"/>
       <c r="P499" s="2" t="n"/>
+      <c r="Q499" s="2" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="2" t="n"/>
@@ -16721,6 +17238,7 @@
       <c r="N500" s="2" t="n"/>
       <c r="O500" s="2" t="n"/>
       <c r="P500" s="2" t="n"/>
+      <c r="Q500" s="2" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="2" t="n"/>
@@ -16753,9 +17271,10 @@
       <c r="N501" s="2" t="n"/>
       <c r="O501" s="2" t="n"/>
       <c r="P501" s="2" t="n"/>
+      <c r="Q501" s="2" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation sqref="E2:E501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown." type="list">
       <formula1>=ChallengeStates</formula1>
     </dataValidation>
@@ -16779,6 +17298,9 @@
     </dataValidation>
     <dataValidation sqref="P2:P501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the dropdown." type="list">
       <formula1>=BonusModes</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q2:Q501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Enter a whole number greater than or equal to 0." type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>